<commit_message>
Redesign task categories for factory director role
Replace generic categories with 6 role-specific ones:
① 経営・対外業務 ② 社内マネジメント ③ 現場管理・監督
④ 現場直接作業 ⑤ 社内事務・管理 ⑥ 定常・移動・休憩

https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録_2026-05-12.xlsx
+++ b/業務記録_2026-05-12.xlsx
@@ -359,7 +359,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="22">
     <font>
       <name val="游ゴシック"/>
       <family val="2"/>
@@ -391,16 +391,87 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="14"/>
     </font>
     <font>
-      <color rgb="00000000"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FF9900"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="00444444"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00375623"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C55A11"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="002E4057"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00595959"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="00FF9900"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="00375623"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="001F4E79"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="00C55A11"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="002E4057"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="00595959"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <color rgb="00000000"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="20">
     <fill>
       <patternFill/>
     </fill>
@@ -451,38 +522,62 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+        <bgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="002F75B6"/>
         <bgColor rgb="002F75B6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004472C4"/>
-        <bgColor rgb="004472C4"/>
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8F4FF"/>
-        <bgColor rgb="00E8F4FF"/>
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFE8E8"/>
-        <bgColor rgb="00FFE8E8"/>
+        <fgColor rgb="00DDEBF7"/>
+        <bgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFB3B3"/>
-        <bgColor rgb="00FFB3B3"/>
+        <fgColor rgb="00FCE4D6"/>
+        <bgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00B3D9FF"/>
-        <bgColor rgb="00B3D9FF"/>
+        <fgColor rgb="00EDF2F9"/>
+        <bgColor rgb="00EDF2F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+        <bgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7F7F7"/>
+        <bgColor rgb="00F7F7F7"/>
       </patternFill>
     </fill>
     <fill>
@@ -870,7 +965,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -1008,10 +1103,100 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="16" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="16" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1019,36 +1204,46 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="15" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -10684,16 +10879,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U47"/>
+  <dimension ref="B2:G45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.875" defaultRowHeight="18.75"/>
   <cols>
     <col width="13.375" customWidth="1" min="1" max="1"/>
-    <col width="17.875" customWidth="1" min="2" max="2"/>
-    <col width="14.625" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="6.125" customWidth="1" min="5" max="5"/>
-    <col width="2.125" customWidth="1" min="6" max="6"/>
-    <col width="5.5" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
     <col width="11.625" customWidth="1" min="8" max="8"/>
     <col width="12.125" customWidth="1" min="9" max="9"/>
     <col width="9.625" customWidth="1" min="10" max="10"/>
@@ -10701,1455 +10896,527 @@
     <col width="7.125" customWidth="1" min="18" max="20"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
-      <c r="R1" s="1" t="n"/>
-      <c r="S1" s="1" t="n"/>
-      <c r="T1" s="1" t="n"/>
-    </row>
-    <row r="2" ht="57" customHeight="1" thickBot="1">
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="3" t="inlineStr">
+    <row r="2" ht="28" customHeight="1" thickBot="1">
+      <c r="B2" s="51" t="inlineStr">
+        <is>
+          <t>取締役工場長　業務記録フォーマット</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="19.5" customHeight="1" thickBot="1"/>
+    <row r="4" ht="20" customHeight="1" thickBot="1">
+      <c r="B4" s="52" t="inlineStr">
+        <is>
+          <t>【カテゴリ定義】</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="B5" s="52" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C5" s="52" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D5" s="52" t="inlineStr">
+        <is>
+          <t>業務内容の例</t>
+        </is>
+      </c>
+      <c r="E5" s="53" t="n"/>
+      <c r="F5" s="53" t="n"/>
+      <c r="G5" s="53" t="n"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="B6" s="54" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C6" s="55" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D6" s="56" t="inlineStr">
+        <is>
+          <t>来客対応、銀行・取引先折衝、対外打ち合わせ</t>
+        </is>
+      </c>
+      <c r="E6" s="57" t="n"/>
+      <c r="F6" s="57" t="n"/>
+      <c r="G6" s="57" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="B7" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C7" s="59" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D7" s="60" t="inlineStr">
+        <is>
+          <t>部下・他部門との打ち合わせ、指示・調整</t>
+        </is>
+      </c>
+      <c r="E7" s="61" t="n"/>
+      <c r="F7" s="61" t="n"/>
+      <c r="G7" s="61" t="n"/>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="B8" s="62" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C8" s="63" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D8" s="64" t="inlineStr">
+        <is>
+          <t>現場巡回、品質・安全確認、現場指導</t>
+        </is>
+      </c>
+      <c r="E8" s="65" t="n"/>
+      <c r="F8" s="65" t="n"/>
+      <c r="G8" s="65" t="n"/>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="B9" s="66" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C9" s="67" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D9" s="68" t="inlineStr">
+        <is>
+          <t>自ら手を動かす作業（委任検討対象）</t>
+        </is>
+      </c>
+      <c r="E9" s="69" t="n"/>
+      <c r="F9" s="69" t="n"/>
+      <c r="G9" s="69" t="n"/>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="B10" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C10" s="71" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D10" s="72" t="inlineStr">
+        <is>
+          <t>メール、資料・報告書作成、事務処理</t>
+        </is>
+      </c>
+      <c r="E10" s="73" t="n"/>
+      <c r="F10" s="73" t="n"/>
+      <c r="G10" s="73" t="n"/>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="B11" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C11" s="75" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D11" s="76" t="inlineStr">
+        <is>
+          <t>朝礼、移動、掃除、休憩</t>
+        </is>
+      </c>
+      <c r="E11" s="77" t="n"/>
+      <c r="F11" s="77" t="n"/>
+      <c r="G11" s="77" t="n"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="B14" s="52" t="inlineStr">
+        <is>
+          <t>【日次入力テンプレート】　　日付：</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="B15" s="52" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C15" s="52" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D15" s="52" t="inlineStr">
         <is>
           <t>業務内容</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>業務
-時間
-（h）</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G2" s="6" t="inlineStr">
-        <is>
-          <t>単位</t>
-        </is>
-      </c>
-      <c r="H2" s="7" t="inlineStr">
-        <is>
-          <t>１ヵ月あたりの時間
-(h）</t>
-        </is>
-      </c>
-      <c r="I2" s="8" t="n"/>
-      <c r="R2" s="1" t="n"/>
-      <c r="S2" s="1" t="n"/>
-      <c r="T2" s="1" t="n"/>
-    </row>
-    <row r="3" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B3" s="40" t="inlineStr">
-        <is>
-          <t>削減可能業務</t>
-        </is>
-      </c>
-      <c r="C3" s="9" t="inlineStr">
-        <is>
-          <t>非定常業務</t>
-        </is>
-      </c>
-      <c r="D3" s="10" t="n"/>
-      <c r="E3" s="11" t="n"/>
-      <c r="F3" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G3" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H3" s="41">
-        <f>I3*E3</f>
-        <v/>
-      </c>
-      <c r="I3" s="15">
-        <f>IF(G3="月",$R$4,IF(G3="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="K3" s="20" t="inlineStr">
-        <is>
-          <t>削減可能業務</t>
-        </is>
-      </c>
-      <c r="L3">
-        <f>SUM(H3:H14)</f>
-        <v/>
-      </c>
-      <c r="R3" s="44" t="inlineStr">
-        <is>
-          <t>掛け数</t>
-        </is>
-      </c>
-      <c r="S3" s="51" t="n"/>
-      <c r="T3" s="52" t="n"/>
-    </row>
-    <row r="4" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B4" s="53" t="n"/>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>非定常業務</t>
-        </is>
-      </c>
-      <c r="D4" s="10" t="n"/>
-      <c r="E4" s="11" t="n"/>
-      <c r="F4" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G4" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H4" s="41">
-        <f>I4*E4</f>
-        <v/>
-      </c>
-      <c r="I4" s="15">
-        <f>IF(G4="月",$R$4,IF(G4="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="K4" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">付帯業務　</t>
-        </is>
-      </c>
-      <c r="L4">
-        <f>SUM(H15:H30)</f>
-        <v/>
-      </c>
-      <c r="R4" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="S4" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="T4" s="24" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" s="53" t="n"/>
-      <c r="C5" s="9" t="inlineStr">
-        <is>
-          <t>非定常業務</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="n"/>
-      <c r="E5" s="11" t="n"/>
-      <c r="F5" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G5" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H5" s="41">
-        <f>I5*E5</f>
-        <v/>
-      </c>
-      <c r="I5" s="15">
-        <f>IF(G5="月",$R$4,IF(G5="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="K5" s="25">
-        <f>C31</f>
-        <v/>
-      </c>
-      <c r="L5">
-        <f>SUM(H31:H41)</f>
-        <v/>
-      </c>
-      <c r="R5" s="1" t="n"/>
-      <c r="S5" s="1" t="n"/>
-      <c r="T5" s="1" t="n"/>
-    </row>
-    <row r="6">
-      <c r="B6" s="53" t="n"/>
-      <c r="C6" s="9" t="inlineStr">
-        <is>
-          <t>非定常業務</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="n"/>
-      <c r="E6" s="11" t="n"/>
-      <c r="F6" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G6" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H6" s="41">
-        <f>I6*E6</f>
-        <v/>
-      </c>
-      <c r="I6" s="15">
-        <f>IF(G6="月",$R$4,IF(G6="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>毎日×20　⇒　１ヵ月あたり</t>
-        </is>
-      </c>
-      <c r="S6" s="1" t="n"/>
-      <c r="T6" s="1" t="n"/>
-    </row>
-    <row r="7">
-      <c r="B7" s="53" t="n"/>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>非定常業務</t>
-        </is>
-      </c>
-      <c r="D7" s="10" t="n"/>
-      <c r="E7" s="11" t="n"/>
-      <c r="F7" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G7" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H7" s="41">
-        <f>I7*E7</f>
-        <v/>
-      </c>
-      <c r="I7" s="15">
-        <f>IF(G7="月",$R$4,IF(G7="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>１週間あたりk×4  ⇒　１ヵ月あたり</t>
-        </is>
-      </c>
-      <c r="S7" s="1" t="n"/>
-      <c r="T7" s="1" t="n"/>
-    </row>
-    <row r="8">
-      <c r="B8" s="53" t="n"/>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>非定常業務</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="n"/>
-      <c r="E8" s="11" t="n"/>
-      <c r="F8" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G8" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H8" s="41">
-        <f>I8*E8</f>
-        <v/>
-      </c>
-      <c r="I8" s="15">
-        <f>IF(G8="月",$R$4,IF(G8="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R8" s="1" t="n"/>
-      <c r="S8" s="1" t="n"/>
-      <c r="T8" s="1" t="n"/>
-    </row>
-    <row r="9">
-      <c r="B9" s="53" t="n"/>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>非定常業務</t>
-        </is>
-      </c>
-      <c r="D9" s="10" t="n"/>
-      <c r="E9" s="11" t="n"/>
-      <c r="F9" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G9" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H9" s="41">
-        <f>I9*E9</f>
-        <v/>
-      </c>
-      <c r="I9" s="15">
-        <f>IF(G9="月",$R$4,IF(G9="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R9" s="1" t="n"/>
-      <c r="S9" s="1" t="n"/>
-      <c r="T9" s="1" t="n"/>
-    </row>
-    <row r="10">
-      <c r="B10" s="53" t="n"/>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>非定常業務</t>
-        </is>
-      </c>
-      <c r="D10" s="10" t="n"/>
-      <c r="E10" s="16" t="n"/>
-      <c r="F10" s="17" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G10" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H10" s="41">
-        <f>I10*E10</f>
-        <v/>
-      </c>
-      <c r="I10" s="15">
-        <f>IF(G10="月",$R$4,IF(G10="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R10" s="1" t="n"/>
-      <c r="S10" s="1" t="n"/>
-      <c r="T10" s="1" t="n"/>
-    </row>
-    <row r="11">
-      <c r="B11" s="53" t="n"/>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>非定常業務</t>
-        </is>
-      </c>
-      <c r="D11" s="10" t="n"/>
-      <c r="E11" s="11" t="n"/>
-      <c r="F11" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G11" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H11" s="41">
-        <f>I11*E11</f>
-        <v/>
-      </c>
-      <c r="I11" s="15">
-        <f>IF(G11="月",$R$4,IF(G11="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R11" s="1" t="n"/>
-      <c r="S11" s="1" t="n"/>
-      <c r="T11" s="1" t="n"/>
-    </row>
-    <row r="12">
-      <c r="B12" s="53" t="n"/>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>非定常業務</t>
-        </is>
-      </c>
-      <c r="D12" s="10" t="n"/>
-      <c r="E12" s="11" t="n"/>
-      <c r="F12" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G12" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H12" s="41">
-        <f>I12*E12</f>
-        <v/>
-      </c>
-      <c r="I12" s="15">
-        <f>IF(G12="月",$R$4,IF(G12="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R12" s="1" t="n"/>
-      <c r="S12" s="1" t="n"/>
-      <c r="T12" s="1" t="n"/>
-    </row>
-    <row r="13">
-      <c r="B13" s="53" t="n"/>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>非定常業務</t>
-        </is>
-      </c>
-      <c r="D13" s="10" t="n"/>
-      <c r="E13" s="11" t="n"/>
-      <c r="F13" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G13" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H13" s="41">
-        <f>I13*E13</f>
-        <v/>
-      </c>
-      <c r="I13" s="15">
-        <f>IF(G13="月",$R$4,IF(G13="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R13" s="1" t="n"/>
-      <c r="S13" s="1" t="n"/>
-      <c r="T13" s="1" t="n"/>
-    </row>
-    <row r="14">
-      <c r="B14" s="54" t="n"/>
-      <c r="C14" s="9" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="11" t="n"/>
-      <c r="F14" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G14" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H14" s="41">
-        <f>I14*E14</f>
-        <v/>
-      </c>
-      <c r="I14" s="15">
-        <f>IF(G14="月",$R$4,IF(G14="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R14" s="1" t="n"/>
-      <c r="S14" s="1" t="n"/>
-      <c r="T14" s="1" t="n"/>
-    </row>
-    <row r="15">
-      <c r="B15" s="42" t="inlineStr">
-        <is>
-          <t>付帯業務
-ノンコア業務</t>
-        </is>
-      </c>
-      <c r="C15" s="18" t="inlineStr">
-        <is>
-          <t>主要外業務</t>
-        </is>
-      </c>
-      <c r="D15" s="10" t="n"/>
-      <c r="E15" s="11" t="n"/>
-      <c r="F15" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G15" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H15" s="43">
-        <f>I15*E15</f>
-        <v/>
-      </c>
-      <c r="I15" s="15">
-        <f>IF(G15="月",$R$4,IF(G15="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="53" t="n"/>
-      <c r="C16" s="18" t="inlineStr">
-        <is>
-          <t>主要外業務</t>
-        </is>
-      </c>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="11" t="n"/>
-      <c r="F16" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G16" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H16" s="43">
-        <f>I16*E16</f>
-        <v/>
-      </c>
-      <c r="I16" s="15">
-        <f>IF(G16="月",$R$4,IF(G16="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="53" t="n"/>
-      <c r="C17" s="18" t="inlineStr">
-        <is>
-          <t>主要外業務</t>
-        </is>
-      </c>
-      <c r="D17" s="10" t="n"/>
-      <c r="E17" s="11" t="n"/>
-      <c r="F17" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G17" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H17" s="43">
-        <f>I17*E17</f>
-        <v/>
-      </c>
-      <c r="I17" s="15">
-        <f>IF(G17="月",$R$4,IF(G17="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="53" t="n"/>
-      <c r="C18" s="18" t="inlineStr">
-        <is>
-          <t>主要外業務</t>
-        </is>
-      </c>
-      <c r="D18" s="10" t="n"/>
-      <c r="E18" s="11" t="n"/>
-      <c r="F18" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G18" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H18" s="43">
-        <f>I18*E18</f>
-        <v/>
-      </c>
-      <c r="I18" s="15">
-        <f>IF(G18="月",$R$4,IF(G18="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="53" t="n"/>
-      <c r="C19" s="18" t="inlineStr">
-        <is>
-          <t>主要外業務</t>
-        </is>
-      </c>
-      <c r="D19" s="26" t="n"/>
-      <c r="E19" s="11" t="n"/>
-      <c r="F19" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G19" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H19" s="43">
-        <f>I19*E19</f>
-        <v/>
-      </c>
-      <c r="I19" s="15">
-        <f>IF(G19="月",$R$4,IF(G19="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="53" t="n"/>
-      <c r="C20" s="18" t="inlineStr">
-        <is>
-          <t>主要外業務</t>
-        </is>
-      </c>
-      <c r="D20" s="26" t="n"/>
-      <c r="E20" s="11" t="n"/>
-      <c r="F20" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G20" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H20" s="43">
-        <f>I20*E20</f>
-        <v/>
-      </c>
-      <c r="I20" s="15">
-        <f>IF(G20="月",$R$4,IF(G20="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R20" s="1" t="n"/>
-      <c r="S20" s="1" t="n"/>
-      <c r="T20" s="1" t="n"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="53" t="n"/>
-      <c r="C21" s="18" t="inlineStr">
-        <is>
-          <t>主要外業務</t>
-        </is>
-      </c>
-      <c r="D21" s="26" t="n"/>
-      <c r="E21" s="16" t="n"/>
-      <c r="F21" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G21" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H21" s="43">
-        <f>I21*E21</f>
-        <v/>
-      </c>
-      <c r="I21" s="15">
-        <f>IF(G21="月",$R$4,IF(G21="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R21" s="1" t="n"/>
-      <c r="S21" s="1" t="n"/>
-      <c r="T21" s="1" t="n"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="53" t="n"/>
-      <c r="C22" s="18" t="inlineStr">
-        <is>
-          <t>主要外業務</t>
-        </is>
-      </c>
-      <c r="D22" s="26" t="n"/>
-      <c r="E22" s="16" t="n"/>
-      <c r="F22" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G22" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H22" s="43">
-        <f>I22*E22</f>
-        <v/>
-      </c>
-      <c r="I22" s="15">
-        <f>IF(G22="月",$R$4,IF(G22="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R22" s="1" t="n"/>
-      <c r="S22" s="1" t="n"/>
-      <c r="T22" s="1" t="n"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="53" t="n"/>
-      <c r="C23" s="18" t="inlineStr">
-        <is>
-          <t>主要外業務</t>
-        </is>
-      </c>
-      <c r="D23" s="26" t="n"/>
-      <c r="E23" s="16" t="n"/>
-      <c r="F23" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G23" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H23" s="43">
-        <f>I23*E23</f>
-        <v/>
-      </c>
-      <c r="I23" s="15">
-        <f>IF(G23="月",$R$4,IF(G23="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R23" s="1" t="n"/>
-      <c r="S23" s="1" t="n"/>
-      <c r="T23" s="1" t="n"/>
-    </row>
-    <row r="24">
-      <c r="B24" s="53" t="n"/>
-      <c r="C24" s="18" t="inlineStr">
-        <is>
-          <t>主要外業務</t>
-        </is>
-      </c>
-      <c r="D24" s="26" t="n"/>
-      <c r="E24" s="16" t="n"/>
-      <c r="F24" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G24" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H24" s="43">
-        <f>I24*E24</f>
-        <v/>
-      </c>
-      <c r="I24" s="15">
-        <f>IF(G24="月",$R$4,IF(G24="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R24" s="1" t="n"/>
-      <c r="S24" s="1" t="n"/>
-      <c r="T24" s="1" t="n"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="53" t="n"/>
-      <c r="C25" s="18" t="inlineStr">
-        <is>
-          <t>主要外業務</t>
-        </is>
-      </c>
-      <c r="D25" s="26" t="n"/>
-      <c r="E25" s="16" t="n"/>
-      <c r="F25" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G25" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H25" s="43">
-        <f>I25*E25</f>
-        <v/>
-      </c>
-      <c r="I25" s="15">
-        <f>IF(G25="月",$R$4,IF(G25="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R25" s="1" t="n"/>
-      <c r="S25" s="1" t="n"/>
-      <c r="T25" s="1" t="n"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="53" t="n"/>
-      <c r="C26" s="18" t="inlineStr">
-        <is>
-          <t>主要外業務</t>
-        </is>
-      </c>
-      <c r="D26" s="26" t="n"/>
-      <c r="E26" s="16" t="n"/>
-      <c r="F26" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G26" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H26" s="43">
-        <f>I26*E26</f>
-        <v/>
-      </c>
-      <c r="I26" s="15">
-        <f>IF(G26="月",$R$4,IF(G26="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R26" s="1" t="n"/>
-      <c r="S26" s="1" t="n"/>
-      <c r="T26" s="1" t="n"/>
-    </row>
-    <row r="27">
-      <c r="B27" s="53" t="n"/>
-      <c r="C27" s="18" t="inlineStr">
-        <is>
-          <t>主要外業務</t>
-        </is>
-      </c>
-      <c r="D27" s="10" t="n"/>
-      <c r="E27" s="11" t="n"/>
-      <c r="F27" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G27" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H27" s="43">
-        <f>I27*E27</f>
-        <v/>
-      </c>
-      <c r="I27" s="15">
-        <f>IF(G27="月",$R$4,IF(G27="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R27" s="1" t="n"/>
-      <c r="S27" s="1" t="n"/>
-      <c r="T27" s="1" t="n"/>
-    </row>
-    <row r="28">
-      <c r="B28" s="53" t="n"/>
-      <c r="C28" s="18" t="inlineStr">
-        <is>
-          <t>主要外業務</t>
-        </is>
-      </c>
-      <c r="D28" s="27" t="n"/>
-      <c r="E28" s="28" t="n"/>
-      <c r="F28" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G28" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H28" s="43">
-        <f>I28*E28</f>
-        <v/>
-      </c>
-      <c r="I28" s="15">
-        <f>IF(G28="月",$R$4,IF(G28="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R28" s="1" t="n"/>
-      <c r="S28" s="1" t="n"/>
-      <c r="T28" s="1" t="n"/>
-    </row>
-    <row r="29">
-      <c r="B29" s="53" t="n"/>
-      <c r="C29" s="18" t="inlineStr">
-        <is>
-          <t>主要外業務</t>
-        </is>
-      </c>
-      <c r="D29" s="26" t="n"/>
-      <c r="E29" s="16" t="n"/>
-      <c r="F29" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G29" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H29" s="43">
-        <f>I29*E29</f>
-        <v/>
-      </c>
-      <c r="I29" s="15">
-        <f>IF(G29="月",$R$4,IF(G29="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R29" s="1" t="n"/>
-      <c r="S29" s="1" t="n"/>
-      <c r="T29" s="1" t="n"/>
-    </row>
-    <row r="30">
-      <c r="B30" s="54" t="n"/>
-      <c r="C30" s="18" t="n"/>
-      <c r="D30" s="26" t="n"/>
-      <c r="E30" s="16" t="n"/>
-      <c r="F30" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G30" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H30" s="43">
-        <f>I30*E30</f>
-        <v/>
-      </c>
-      <c r="I30" s="15">
-        <f>IF(G30="月",$R$4,IF(G30="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R30" s="1" t="n"/>
-      <c r="S30" s="1" t="n"/>
-      <c r="T30" s="1" t="n"/>
-    </row>
-    <row r="31">
-      <c r="B31" s="47" t="inlineStr">
-        <is>
-          <t>主体業務
-コア業務</t>
-        </is>
-      </c>
-      <c r="C31" s="29" t="inlineStr">
-        <is>
-          <t>主体業務</t>
-        </is>
-      </c>
-      <c r="D31" s="10" t="n"/>
-      <c r="E31" s="16" t="n"/>
-      <c r="F31" s="17" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G31" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H31" s="48">
-        <f>I31*E31</f>
-        <v/>
-      </c>
-      <c r="I31" s="15">
-        <f>IF(G31="月",$R$4,IF(G31="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R31" s="1" t="n"/>
-      <c r="S31" s="1" t="n"/>
-      <c r="T31" s="1" t="n"/>
-    </row>
-    <row r="32">
-      <c r="B32" s="53" t="n"/>
-      <c r="C32" s="29" t="inlineStr">
-        <is>
-          <t>主体業務</t>
-        </is>
-      </c>
-      <c r="D32" s="10" t="n"/>
-      <c r="E32" s="11" t="n"/>
-      <c r="F32" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G32" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H32" s="48">
-        <f>I32*E32</f>
-        <v/>
-      </c>
-      <c r="I32" s="15">
-        <f>IF(G32="月",$R$4,IF(G32="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R32" s="1" t="n"/>
-      <c r="S32" s="1" t="n"/>
-      <c r="T32" s="1" t="n"/>
-    </row>
-    <row r="33">
-      <c r="B33" s="53" t="n"/>
-      <c r="C33" s="29" t="inlineStr">
-        <is>
-          <t>主体業務</t>
-        </is>
-      </c>
-      <c r="D33" s="10" t="n"/>
-      <c r="E33" s="11" t="n"/>
-      <c r="F33" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G33" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H33" s="48">
-        <f>I33*E33</f>
-        <v/>
-      </c>
-      <c r="I33" s="15">
-        <f>IF(G33="月",$R$4,IF(G33="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R33" s="1" t="n"/>
-      <c r="S33" s="1" t="n"/>
-      <c r="T33" s="1" t="n"/>
-    </row>
-    <row r="34">
-      <c r="B34" s="53" t="n"/>
-      <c r="C34" s="29" t="inlineStr">
-        <is>
-          <t>主体業務</t>
-        </is>
-      </c>
-      <c r="D34" s="10" t="n"/>
-      <c r="E34" s="11" t="n"/>
-      <c r="F34" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G34" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H34" s="48">
-        <f>I34*E34</f>
-        <v/>
-      </c>
-      <c r="I34" s="15">
-        <f>IF(G34="月",$R$4,IF(G34="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R34" s="1" t="n"/>
-      <c r="S34" s="1" t="n"/>
-      <c r="T34" s="1" t="n"/>
-    </row>
-    <row r="35">
-      <c r="B35" s="53" t="n"/>
-      <c r="C35" s="29" t="inlineStr">
-        <is>
-          <t>主体業務</t>
-        </is>
-      </c>
-      <c r="D35" s="10" t="n"/>
-      <c r="E35" s="11" t="n"/>
-      <c r="F35" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G35" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H35" s="48">
-        <f>I35*E35</f>
-        <v/>
-      </c>
-      <c r="I35" s="15">
-        <f>IF(G35="月",$R$4,IF(G35="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R35" s="1" t="n"/>
-      <c r="S35" s="1" t="n"/>
-      <c r="T35" s="1" t="n"/>
-    </row>
-    <row r="36">
-      <c r="B36" s="53" t="n"/>
-      <c r="C36" s="29" t="inlineStr">
-        <is>
-          <t>主体業務</t>
-        </is>
-      </c>
-      <c r="D36" s="10" t="n"/>
-      <c r="E36" s="11" t="n"/>
-      <c r="F36" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G36" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H36" s="48">
-        <f>I36*E36</f>
-        <v/>
-      </c>
-      <c r="I36" s="15">
-        <f>IF(G36="月",$R$4,IF(G36="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R36" s="1" t="n"/>
-      <c r="S36" s="1" t="n"/>
-      <c r="T36" s="1" t="n"/>
-    </row>
-    <row r="37">
-      <c r="B37" s="53" t="n"/>
-      <c r="C37" s="29" t="inlineStr">
-        <is>
-          <t>主体業務</t>
-        </is>
-      </c>
-      <c r="D37" s="10" t="n"/>
-      <c r="E37" s="11" t="n"/>
-      <c r="F37" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G37" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H37" s="48">
-        <f>I37*E37</f>
-        <v/>
-      </c>
-      <c r="I37" s="15">
-        <f>IF(G37="月",$R$4,IF(G37="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R37" s="1" t="n"/>
-      <c r="S37" s="1" t="n"/>
-      <c r="T37" s="1" t="n"/>
-    </row>
-    <row r="38">
-      <c r="B38" s="53" t="n"/>
-      <c r="C38" s="29" t="inlineStr">
-        <is>
-          <t>主体業務</t>
-        </is>
-      </c>
-      <c r="D38" s="27" t="n"/>
-      <c r="E38" s="28" t="n"/>
-      <c r="F38" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G38" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H38" s="48">
-        <f>I38*E38</f>
-        <v/>
-      </c>
-      <c r="I38" s="15">
-        <f>IF(G38="月",$R$4,IF(G38="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R38" s="1" t="n"/>
-      <c r="S38" s="1" t="n"/>
-      <c r="T38" s="1" t="n"/>
-    </row>
-    <row r="39">
-      <c r="B39" s="53" t="n"/>
-      <c r="C39" s="29" t="inlineStr">
-        <is>
-          <t>主体業務</t>
-        </is>
-      </c>
-      <c r="D39" s="27" t="n"/>
-      <c r="E39" s="28" t="n"/>
-      <c r="F39" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G39" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H39" s="48">
-        <f>I39*E39</f>
-        <v/>
-      </c>
-      <c r="I39" s="15">
-        <f>IF(G39="月",$R$4,IF(G39="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R39" s="1" t="n"/>
-      <c r="S39" s="1" t="n"/>
-      <c r="T39" s="1" t="n"/>
-    </row>
-    <row r="40">
-      <c r="B40" s="53" t="n"/>
-      <c r="C40" s="29" t="inlineStr">
-        <is>
-          <t>主体業務</t>
-        </is>
-      </c>
-      <c r="D40" s="27" t="n"/>
-      <c r="E40" s="28" t="n"/>
-      <c r="F40" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G40" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H40" s="48">
-        <f>I40*E40</f>
-        <v/>
-      </c>
-      <c r="I40" s="15">
-        <f>IF(G40="月",$R$4,IF(G40="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R40" s="1" t="n"/>
-      <c r="S40" s="1" t="n"/>
-      <c r="T40" s="1" t="n"/>
-    </row>
-    <row r="41">
-      <c r="B41" s="53" t="n"/>
-      <c r="C41" s="29" t="inlineStr">
-        <is>
-          <t>主体業務</t>
-        </is>
-      </c>
-      <c r="D41" s="27" t="n"/>
-      <c r="E41" s="28" t="n"/>
-      <c r="F41" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G41" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H41" s="48">
-        <f>I41*E41</f>
-        <v/>
-      </c>
-      <c r="I41" s="15">
-        <f>IF(G41="月",$R$4,IF(G41="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R41" s="1" t="n"/>
-      <c r="S41" s="1" t="n"/>
-      <c r="T41" s="1" t="n"/>
-    </row>
-    <row r="42">
-      <c r="B42" s="53" t="n"/>
-      <c r="C42" s="29" t="inlineStr">
-        <is>
-          <t>主体業務</t>
-        </is>
-      </c>
-      <c r="D42" s="27" t="n"/>
-      <c r="E42" s="28" t="n"/>
-      <c r="F42" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G42" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H42" s="48">
-        <f>I42*E42</f>
-        <v/>
-      </c>
-      <c r="I42" s="15">
-        <f>IF(G42="月",$R$4,IF(G42="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R42" s="1" t="n"/>
-      <c r="S42" s="1" t="n"/>
-      <c r="T42" s="1" t="n"/>
-    </row>
-    <row r="43" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B43" s="54" t="n"/>
-      <c r="C43" s="31" t="n"/>
-      <c r="D43" s="27" t="n"/>
-      <c r="E43" s="28" t="n"/>
-      <c r="F43" s="12" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G43" s="13" t="inlineStr">
-        <is>
-          <t>月</t>
-        </is>
-      </c>
-      <c r="H43" s="48">
-        <f>I43*E43</f>
-        <v/>
-      </c>
-      <c r="I43" s="15">
-        <f>IF(G43="月",$R$4,IF(G43="週",$S$4,$T$4))</f>
-        <v/>
-      </c>
-      <c r="R43" s="1" t="n"/>
-      <c r="S43" s="1" t="n"/>
-      <c r="T43" s="1" t="n"/>
-    </row>
-    <row r="44" ht="24.75" customHeight="1" thickTop="1">
-      <c r="A44" s="32" t="n"/>
-      <c r="B44" s="32" t="n"/>
-      <c r="C44" s="49" t="inlineStr">
+      <c r="E15" s="52" t="inlineStr">
+        <is>
+          <t>開始</t>
+        </is>
+      </c>
+      <c r="F15" s="52" t="inlineStr">
+        <is>
+          <t>終了</t>
+        </is>
+      </c>
+      <c r="G15" s="52" t="inlineStr">
+        <is>
+          <t>所要時間（分）</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="B16" s="78" t="n"/>
+      <c r="C16" s="78" t="n"/>
+      <c r="D16" s="78" t="n"/>
+      <c r="E16" s="78" t="n"/>
+      <c r="F16" s="78" t="n"/>
+      <c r="G16" s="78" t="n"/>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="B17" s="79" t="n"/>
+      <c r="C17" s="79" t="n"/>
+      <c r="D17" s="79" t="n"/>
+      <c r="E17" s="79" t="n"/>
+      <c r="F17" s="79" t="n"/>
+      <c r="G17" s="79" t="n"/>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="B18" s="78" t="n"/>
+      <c r="C18" s="78" t="n"/>
+      <c r="D18" s="78" t="n"/>
+      <c r="E18" s="78" t="n"/>
+      <c r="F18" s="78" t="n"/>
+      <c r="G18" s="78" t="n"/>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="B19" s="79" t="n"/>
+      <c r="C19" s="79" t="n"/>
+      <c r="D19" s="79" t="n"/>
+      <c r="E19" s="79" t="n"/>
+      <c r="F19" s="79" t="n"/>
+      <c r="G19" s="79" t="n"/>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="B20" s="78" t="n"/>
+      <c r="C20" s="78" t="n"/>
+      <c r="D20" s="78" t="n"/>
+      <c r="E20" s="78" t="n"/>
+      <c r="F20" s="78" t="n"/>
+      <c r="G20" s="78" t="n"/>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="B21" s="79" t="n"/>
+      <c r="C21" s="79" t="n"/>
+      <c r="D21" s="79" t="n"/>
+      <c r="E21" s="79" t="n"/>
+      <c r="F21" s="79" t="n"/>
+      <c r="G21" s="79" t="n"/>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="B22" s="78" t="n"/>
+      <c r="C22" s="78" t="n"/>
+      <c r="D22" s="78" t="n"/>
+      <c r="E22" s="78" t="n"/>
+      <c r="F22" s="78" t="n"/>
+      <c r="G22" s="78" t="n"/>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="B23" s="79" t="n"/>
+      <c r="C23" s="79" t="n"/>
+      <c r="D23" s="79" t="n"/>
+      <c r="E23" s="79" t="n"/>
+      <c r="F23" s="79" t="n"/>
+      <c r="G23" s="79" t="n"/>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="B24" s="78" t="n"/>
+      <c r="C24" s="78" t="n"/>
+      <c r="D24" s="78" t="n"/>
+      <c r="E24" s="78" t="n"/>
+      <c r="F24" s="78" t="n"/>
+      <c r="G24" s="78" t="n"/>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="B25" s="79" t="n"/>
+      <c r="C25" s="79" t="n"/>
+      <c r="D25" s="79" t="n"/>
+      <c r="E25" s="79" t="n"/>
+      <c r="F25" s="79" t="n"/>
+      <c r="G25" s="79" t="n"/>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="B26" s="78" t="n"/>
+      <c r="C26" s="78" t="n"/>
+      <c r="D26" s="78" t="n"/>
+      <c r="E26" s="78" t="n"/>
+      <c r="F26" s="78" t="n"/>
+      <c r="G26" s="78" t="n"/>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="B27" s="79" t="n"/>
+      <c r="C27" s="79" t="n"/>
+      <c r="D27" s="79" t="n"/>
+      <c r="E27" s="79" t="n"/>
+      <c r="F27" s="79" t="n"/>
+      <c r="G27" s="79" t="n"/>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="B28" s="78" t="n"/>
+      <c r="C28" s="78" t="n"/>
+      <c r="D28" s="78" t="n"/>
+      <c r="E28" s="78" t="n"/>
+      <c r="F28" s="78" t="n"/>
+      <c r="G28" s="78" t="n"/>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="B29" s="79" t="n"/>
+      <c r="C29" s="79" t="n"/>
+      <c r="D29" s="79" t="n"/>
+      <c r="E29" s="79" t="n"/>
+      <c r="F29" s="79" t="n"/>
+      <c r="G29" s="79" t="n"/>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="B30" s="78" t="n"/>
+      <c r="C30" s="78" t="n"/>
+      <c r="D30" s="78" t="n"/>
+      <c r="E30" s="78" t="n"/>
+      <c r="F30" s="78" t="n"/>
+      <c r="G30" s="78" t="n"/>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="B31" s="79" t="n"/>
+      <c r="C31" s="79" t="n"/>
+      <c r="D31" s="79" t="n"/>
+      <c r="E31" s="79" t="n"/>
+      <c r="F31" s="79" t="n"/>
+      <c r="G31" s="79" t="n"/>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="B32" s="78" t="n"/>
+      <c r="C32" s="78" t="n"/>
+      <c r="D32" s="78" t="n"/>
+      <c r="E32" s="78" t="n"/>
+      <c r="F32" s="78" t="n"/>
+      <c r="G32" s="78" t="n"/>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="B33" s="79" t="n"/>
+      <c r="C33" s="79" t="n"/>
+      <c r="D33" s="79" t="n"/>
+      <c r="E33" s="79" t="n"/>
+      <c r="F33" s="79" t="n"/>
+      <c r="G33" s="79" t="n"/>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="B34" s="78" t="n"/>
+      <c r="C34" s="78" t="n"/>
+      <c r="D34" s="78" t="n"/>
+      <c r="E34" s="78" t="n"/>
+      <c r="F34" s="78" t="n"/>
+      <c r="G34" s="78" t="n"/>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="B35" s="79" t="n"/>
+      <c r="C35" s="79" t="n"/>
+      <c r="D35" s="79" t="n"/>
+      <c r="E35" s="79" t="n"/>
+      <c r="F35" s="79" t="n"/>
+      <c r="G35" s="79" t="n"/>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="B37" s="52" t="inlineStr">
+        <is>
+          <t>【カテゴリ別集計】</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="B38" s="52" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C38" s="52" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D38" s="52" t="inlineStr">
+        <is>
+          <t>合計（分）</t>
+        </is>
+      </c>
+      <c r="E38" s="52" t="inlineStr">
+        <is>
+          <t>合計（時間）</t>
+        </is>
+      </c>
+      <c r="F38" s="52" t="inlineStr">
+        <is>
+          <t>割合</t>
+        </is>
+      </c>
+      <c r="G38" s="52" t="inlineStr">
+        <is>
+          <t>評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="B39" s="54" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C39" s="80" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D39" s="57" t="n"/>
+      <c r="E39" s="57" t="n"/>
+      <c r="F39" s="57" t="n"/>
+      <c r="G39" s="57" t="n"/>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="B40" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C40" s="81" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D40" s="61" t="n"/>
+      <c r="E40" s="61" t="n"/>
+      <c r="F40" s="61" t="n"/>
+      <c r="G40" s="61" t="n"/>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="B41" s="62" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C41" s="82" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D41" s="65" t="n"/>
+      <c r="E41" s="65" t="n"/>
+      <c r="F41" s="65" t="n"/>
+      <c r="G41" s="65" t="n"/>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="B42" s="66" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C42" s="83" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D42" s="69" t="n"/>
+      <c r="E42" s="69" t="n"/>
+      <c r="F42" s="69" t="n"/>
+      <c r="G42" s="69" t="n"/>
+    </row>
+    <row r="43" ht="18" customHeight="1" thickBot="1">
+      <c r="B43" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C43" s="84" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D43" s="73" t="n"/>
+      <c r="E43" s="73" t="n"/>
+      <c r="F43" s="73" t="n"/>
+      <c r="G43" s="73" t="n"/>
+    </row>
+    <row r="44" ht="18" customHeight="1" thickTop="1">
+      <c r="B44" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C44" s="85" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D44" s="77" t="n"/>
+      <c r="E44" s="77" t="n"/>
+      <c r="F44" s="77" t="n"/>
+      <c r="G44" s="77" t="n"/>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="B45" s="86" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="D44" s="55" t="n"/>
-      <c r="E44" s="55" t="n"/>
-      <c r="F44" s="55" t="n"/>
-      <c r="G44" s="56" t="n"/>
-      <c r="H44" s="33">
-        <f>SUM(H3:H43)</f>
-        <v/>
-      </c>
-      <c r="I44" s="34" t="n"/>
-      <c r="J44" s="32" t="n"/>
-      <c r="K44" s="32" t="n"/>
-      <c r="L44" s="32" t="n"/>
-      <c r="M44" s="32" t="n"/>
-      <c r="N44" s="32" t="n"/>
-      <c r="O44" s="32" t="n"/>
-      <c r="P44" s="32" t="n"/>
-      <c r="Q44" s="32" t="n"/>
-      <c r="R44" s="34" t="n"/>
-      <c r="S44" s="34" t="n"/>
-      <c r="T44" s="34" t="n"/>
-      <c r="U44" s="32" t="n"/>
-    </row>
-    <row r="45" ht="24" customHeight="1">
-      <c r="A45" s="32" t="n"/>
-      <c r="B45" s="32" t="n"/>
-      <c r="C45" s="50" t="inlineStr">
-        <is>
-          <t>実際の勤務時間</t>
-        </is>
-      </c>
-      <c r="D45" s="57" t="n"/>
-      <c r="E45" s="57" t="n"/>
-      <c r="F45" s="57" t="n"/>
-      <c r="G45" s="58" t="n"/>
-      <c r="H45" s="50" t="n"/>
-      <c r="I45" s="36" t="n"/>
-      <c r="J45" s="32" t="n"/>
-      <c r="K45" s="32" t="n"/>
-      <c r="L45" s="32" t="n"/>
-      <c r="M45" s="32" t="n"/>
-      <c r="N45" s="32" t="n"/>
-      <c r="O45" s="32" t="n"/>
-      <c r="P45" s="32" t="n"/>
-      <c r="Q45" s="32" t="n"/>
-      <c r="R45" s="36" t="n"/>
-      <c r="S45" s="36" t="n"/>
-      <c r="T45" s="36" t="n"/>
-      <c r="U45" s="32" t="n"/>
-    </row>
-    <row r="46" ht="24" customHeight="1">
-      <c r="A46" s="32" t="n"/>
-      <c r="B46" s="32" t="n"/>
-      <c r="C46" s="39" t="inlineStr">
-        <is>
-          <t>比率</t>
-        </is>
-      </c>
-      <c r="D46" s="57" t="n"/>
-      <c r="E46" s="57" t="n"/>
-      <c r="F46" s="57" t="n"/>
-      <c r="G46" s="58" t="n"/>
-      <c r="H46" s="37">
-        <f>H44/H45</f>
-        <v/>
-      </c>
-      <c r="I46" s="59" t="n"/>
-      <c r="J46" s="32" t="n"/>
-      <c r="K46" s="32" t="n"/>
-      <c r="L46" s="32" t="n"/>
-      <c r="M46" s="32" t="n"/>
-      <c r="N46" s="32" t="n"/>
-      <c r="O46" s="32" t="n"/>
-      <c r="P46" s="32" t="n"/>
-      <c r="Q46" s="32" t="n"/>
-      <c r="R46" s="59" t="n"/>
-      <c r="S46" s="59" t="n"/>
-      <c r="T46" s="59" t="n"/>
-      <c r="U46" s="32" t="n"/>
-    </row>
-    <row r="47">
-      <c r="E47" s="1" t="n"/>
-      <c r="F47" s="1" t="n"/>
-      <c r="G47" s="1" t="n"/>
-      <c r="R47" s="1" t="n"/>
-      <c r="S47" s="1" t="n"/>
-      <c r="T47" s="1" t="n"/>
-    </row>
+      <c r="C45" s="86" t="n"/>
+      <c r="D45" s="86" t="n"/>
+      <c r="E45" s="86" t="n"/>
+      <c r="F45" s="86" t="n"/>
+      <c r="G45" s="86" t="n"/>
+    </row>
+    <row r="46" ht="24" customHeight="1"/>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="17">
     <mergeCell ref="B31:B43"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="E10:G10"/>
     <mergeCell ref="R3:T3"/>
+    <mergeCell ref="E11:G11"/>
     <mergeCell ref="C46:G46"/>
+    <mergeCell ref="B14:G14"/>
+    <mergeCell ref="B37:G37"/>
+    <mergeCell ref="E8:G8"/>
     <mergeCell ref="C44:G44"/>
+    <mergeCell ref="B4:G4"/>
+    <mergeCell ref="E9:G9"/>
     <mergeCell ref="C45:G45"/>
     <mergeCell ref="B3:B14"/>
     <mergeCell ref="B15:B30"/>
+    <mergeCell ref="E7:G7"/>
+    <mergeCell ref="E6:G6"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="G3:G43" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
@@ -12269,7 +11536,7 @@
       </c>
     </row>
     <row r="4" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B4" s="53" t="n"/>
+      <c r="B4" s="87" t="n"/>
       <c r="C4" s="9" t="inlineStr">
         <is>
           <t>非定常業務</t>
@@ -12303,7 +11570,7 @@
       </c>
     </row>
     <row r="5" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B5" s="53" t="n"/>
+      <c r="B5" s="87" t="n"/>
       <c r="C5" s="9" t="inlineStr">
         <is>
           <t>非定常業務</t>
@@ -12331,7 +11598,7 @@
       </c>
     </row>
     <row r="6" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B6" s="53" t="n"/>
+      <c r="B6" s="87" t="n"/>
       <c r="C6" s="9" t="inlineStr">
         <is>
           <t>非定常業務</t>
@@ -12359,7 +11626,7 @@
       </c>
     </row>
     <row r="7" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B7" s="53" t="n"/>
+      <c r="B7" s="87" t="n"/>
       <c r="C7" s="9" t="inlineStr">
         <is>
           <t>非定常業務</t>
@@ -12387,7 +11654,7 @@
       </c>
     </row>
     <row r="8" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B8" s="53" t="n"/>
+      <c r="B8" s="87" t="n"/>
       <c r="C8" s="9" t="inlineStr">
         <is>
           <t>非定常業務</t>
@@ -12418,7 +11685,7 @@
       <c r="T8" s="1" t="n"/>
     </row>
     <row r="9" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B9" s="53" t="n"/>
+      <c r="B9" s="87" t="n"/>
       <c r="C9" s="9" t="inlineStr">
         <is>
           <t>非定常業務</t>
@@ -12449,7 +11716,7 @@
       <c r="T9" s="1" t="n"/>
     </row>
     <row r="10" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B10" s="53" t="n"/>
+      <c r="B10" s="87" t="n"/>
       <c r="C10" s="9" t="inlineStr">
         <is>
           <t>非定常業務</t>
@@ -12480,7 +11747,7 @@
       <c r="T10" s="1" t="n"/>
     </row>
     <row r="11" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B11" s="53" t="n"/>
+      <c r="B11" s="87" t="n"/>
       <c r="C11" s="9" t="inlineStr">
         <is>
           <t>非定常業務</t>
@@ -12511,7 +11778,7 @@
       <c r="T11" s="1" t="n"/>
     </row>
     <row r="12" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B12" s="53" t="n"/>
+      <c r="B12" s="87" t="n"/>
       <c r="C12" s="9" t="inlineStr">
         <is>
           <t>非定常業務</t>
@@ -12542,7 +11809,7 @@
       <c r="T12" s="1" t="n"/>
     </row>
     <row r="13" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B13" s="53" t="n"/>
+      <c r="B13" s="87" t="n"/>
       <c r="C13" s="9" t="inlineStr">
         <is>
           <t>非定常業務</t>
@@ -12573,7 +11840,7 @@
       <c r="T13" s="1" t="n"/>
     </row>
     <row r="14" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B14" s="54" t="n"/>
+      <c r="B14" s="88" t="n"/>
       <c r="C14" s="9" t="n"/>
       <c r="D14" s="10" t="n"/>
       <c r="E14" s="11" t="n"/>
@@ -12651,11 +11918,11 @@
           <t>掛け数</t>
         </is>
       </c>
-      <c r="S15" s="51" t="n"/>
-      <c r="T15" s="52" t="n"/>
+      <c r="S15" s="89" t="n"/>
+      <c r="T15" s="90" t="n"/>
     </row>
     <row r="16" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B16" s="53" t="n"/>
+      <c r="B16" s="87" t="n"/>
       <c r="C16" s="18" t="inlineStr">
         <is>
           <t>主要外業務</t>
@@ -12707,7 +11974,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="53" t="n"/>
+      <c r="B17" s="87" t="n"/>
       <c r="C17" s="18" t="inlineStr">
         <is>
           <t>主要外業務</t>
@@ -12752,7 +12019,7 @@
       <c r="T17" s="1" t="n"/>
     </row>
     <row r="18">
-      <c r="B18" s="53" t="n"/>
+      <c r="B18" s="87" t="n"/>
       <c r="C18" s="18" t="inlineStr">
         <is>
           <t>主要外業務</t>
@@ -12793,7 +12060,7 @@
       <c r="T18" s="1" t="n"/>
     </row>
     <row r="19">
-      <c r="B19" s="53" t="n"/>
+      <c r="B19" s="87" t="n"/>
       <c r="C19" s="18" t="inlineStr">
         <is>
           <t>主要外業務</t>
@@ -12834,7 +12101,7 @@
       <c r="T19" s="1" t="n"/>
     </row>
     <row r="20">
-      <c r="B20" s="53" t="n"/>
+      <c r="B20" s="87" t="n"/>
       <c r="C20" s="18" t="inlineStr">
         <is>
           <t>主要外業務</t>
@@ -12871,7 +12138,7 @@
       <c r="T20" s="1" t="n"/>
     </row>
     <row r="21">
-      <c r="B21" s="53" t="n"/>
+      <c r="B21" s="87" t="n"/>
       <c r="C21" s="18" t="inlineStr">
         <is>
           <t>主要外業務</t>
@@ -12908,7 +12175,7 @@
       <c r="T21" s="1" t="n"/>
     </row>
     <row r="22" hidden="1">
-      <c r="B22" s="53" t="n"/>
+      <c r="B22" s="87" t="n"/>
       <c r="C22" s="18" t="inlineStr">
         <is>
           <t>主要外業務</t>
@@ -12939,7 +12206,7 @@
       <c r="T22" s="1" t="n"/>
     </row>
     <row r="23" hidden="1">
-      <c r="B23" s="53" t="n"/>
+      <c r="B23" s="87" t="n"/>
       <c r="C23" s="18" t="inlineStr">
         <is>
           <t>主要外業務</t>
@@ -12970,7 +12237,7 @@
       <c r="T23" s="1" t="n"/>
     </row>
     <row r="24" hidden="1">
-      <c r="B24" s="53" t="n"/>
+      <c r="B24" s="87" t="n"/>
       <c r="C24" s="18" t="inlineStr">
         <is>
           <t>主要外業務</t>
@@ -13001,7 +12268,7 @@
       <c r="T24" s="1" t="n"/>
     </row>
     <row r="25" hidden="1">
-      <c r="B25" s="53" t="n"/>
+      <c r="B25" s="87" t="n"/>
       <c r="C25" s="18" t="inlineStr">
         <is>
           <t>主要外業務</t>
@@ -13032,7 +12299,7 @@
       <c r="T25" s="1" t="n"/>
     </row>
     <row r="26" hidden="1">
-      <c r="B26" s="53" t="n"/>
+      <c r="B26" s="87" t="n"/>
       <c r="C26" s="18" t="inlineStr">
         <is>
           <t>主要外業務</t>
@@ -13063,7 +12330,7 @@
       <c r="T26" s="1" t="n"/>
     </row>
     <row r="27" hidden="1">
-      <c r="B27" s="53" t="n"/>
+      <c r="B27" s="87" t="n"/>
       <c r="C27" s="18" t="inlineStr">
         <is>
           <t>主要外業務</t>
@@ -13094,7 +12361,7 @@
       <c r="T27" s="1" t="n"/>
     </row>
     <row r="28" hidden="1">
-      <c r="B28" s="53" t="n"/>
+      <c r="B28" s="87" t="n"/>
       <c r="C28" s="18" t="inlineStr">
         <is>
           <t>主要外業務</t>
@@ -13125,7 +12392,7 @@
       <c r="T28" s="1" t="n"/>
     </row>
     <row r="29" hidden="1">
-      <c r="B29" s="53" t="n"/>
+      <c r="B29" s="87" t="n"/>
       <c r="C29" s="18" t="inlineStr">
         <is>
           <t>主要外業務</t>
@@ -13156,7 +12423,7 @@
       <c r="T29" s="1" t="n"/>
     </row>
     <row r="30" hidden="1">
-      <c r="B30" s="54" t="n"/>
+      <c r="B30" s="88" t="n"/>
       <c r="C30" s="18" t="n"/>
       <c r="D30" s="26" t="n"/>
       <c r="E30" s="16" t="n"/>
@@ -13225,7 +12492,7 @@
       <c r="T31" s="1" t="n"/>
     </row>
     <row r="32">
-      <c r="B32" s="53" t="n"/>
+      <c r="B32" s="87" t="n"/>
       <c r="C32" s="29" t="inlineStr">
         <is>
           <t>主体業務</t>
@@ -13262,7 +12529,7 @@
       <c r="T32" s="1" t="n"/>
     </row>
     <row r="33" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B33" s="53" t="n"/>
+      <c r="B33" s="87" t="n"/>
       <c r="C33" s="29" t="inlineStr">
         <is>
           <t>主体業務</t>
@@ -13299,7 +12566,7 @@
       <c r="T33" s="1" t="n"/>
     </row>
     <row r="34" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B34" s="53" t="n"/>
+      <c r="B34" s="87" t="n"/>
       <c r="C34" s="29" t="inlineStr">
         <is>
           <t>主体業務</t>
@@ -13330,7 +12597,7 @@
       <c r="T34" s="1" t="n"/>
     </row>
     <row r="35" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B35" s="53" t="n"/>
+      <c r="B35" s="87" t="n"/>
       <c r="C35" s="29" t="inlineStr">
         <is>
           <t>主体業務</t>
@@ -13361,7 +12628,7 @@
       <c r="T35" s="1" t="n"/>
     </row>
     <row r="36" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B36" s="53" t="n"/>
+      <c r="B36" s="87" t="n"/>
       <c r="C36" s="29" t="inlineStr">
         <is>
           <t>主体業務</t>
@@ -13392,7 +12659,7 @@
       <c r="T36" s="1" t="n"/>
     </row>
     <row r="37" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B37" s="53" t="n"/>
+      <c r="B37" s="87" t="n"/>
       <c r="C37" s="29" t="inlineStr">
         <is>
           <t>主体業務</t>
@@ -13423,7 +12690,7 @@
       <c r="T37" s="1" t="n"/>
     </row>
     <row r="38" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B38" s="53" t="n"/>
+      <c r="B38" s="87" t="n"/>
       <c r="C38" s="29" t="inlineStr">
         <is>
           <t>主体業務</t>
@@ -13454,7 +12721,7 @@
       <c r="T38" s="1" t="n"/>
     </row>
     <row r="39" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B39" s="53" t="n"/>
+      <c r="B39" s="87" t="n"/>
       <c r="C39" s="29" t="inlineStr">
         <is>
           <t>主体業務</t>
@@ -13485,7 +12752,7 @@
       <c r="T39" s="1" t="n"/>
     </row>
     <row r="40" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B40" s="53" t="n"/>
+      <c r="B40" s="87" t="n"/>
       <c r="C40" s="29" t="inlineStr">
         <is>
           <t>主体業務</t>
@@ -13516,7 +12783,7 @@
       <c r="T40" s="1" t="n"/>
     </row>
     <row r="41" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B41" s="53" t="n"/>
+      <c r="B41" s="87" t="n"/>
       <c r="C41" s="29" t="inlineStr">
         <is>
           <t>主体業務</t>
@@ -13547,7 +12814,7 @@
       <c r="T41" s="1" t="n"/>
     </row>
     <row r="42" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B42" s="53" t="n"/>
+      <c r="B42" s="87" t="n"/>
       <c r="C42" s="29" t="inlineStr">
         <is>
           <t>主体業務</t>
@@ -13578,7 +12845,7 @@
       <c r="T42" s="1" t="n"/>
     </row>
     <row r="43" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B43" s="54" t="n"/>
+      <c r="B43" s="88" t="n"/>
       <c r="C43" s="31" t="n"/>
       <c r="D43" s="27" t="n"/>
       <c r="E43" s="28" t="n"/>
@@ -13612,10 +12879,10 @@
           <t>合計</t>
         </is>
       </c>
-      <c r="D44" s="55" t="n"/>
-      <c r="E44" s="55" t="n"/>
-      <c r="F44" s="55" t="n"/>
-      <c r="G44" s="56" t="n"/>
+      <c r="D44" s="91" t="n"/>
+      <c r="E44" s="91" t="n"/>
+      <c r="F44" s="91" t="n"/>
+      <c r="G44" s="92" t="n"/>
       <c r="H44" s="33">
         <f>SUM(H3:H43)</f>
         <v/>
@@ -13642,10 +12909,10 @@
           <t>実際の勤務時間</t>
         </is>
       </c>
-      <c r="D45" s="57" t="n"/>
-      <c r="E45" s="57" t="n"/>
-      <c r="F45" s="57" t="n"/>
-      <c r="G45" s="58" t="n"/>
+      <c r="D45" s="93" t="n"/>
+      <c r="E45" s="93" t="n"/>
+      <c r="F45" s="93" t="n"/>
+      <c r="G45" s="94" t="n"/>
       <c r="H45" s="50" t="n">
         <v>9.66</v>
       </c>
@@ -13671,15 +12938,15 @@
           <t>比率</t>
         </is>
       </c>
-      <c r="D46" s="57" t="n"/>
-      <c r="E46" s="57" t="n"/>
-      <c r="F46" s="57" t="n"/>
-      <c r="G46" s="58" t="n"/>
+      <c r="D46" s="93" t="n"/>
+      <c r="E46" s="93" t="n"/>
+      <c r="F46" s="93" t="n"/>
+      <c r="G46" s="94" t="n"/>
       <c r="H46" s="37">
         <f>H44/H45</f>
         <v/>
       </c>
-      <c r="I46" s="59" t="n"/>
+      <c r="I46" s="95" t="n"/>
       <c r="J46" s="32" t="n"/>
       <c r="K46" s="32" t="n"/>
       <c r="L46" s="32" t="n"/>
@@ -13688,9 +12955,9 @@
       <c r="O46" s="32" t="n"/>
       <c r="P46" s="32" t="n"/>
       <c r="Q46" s="32" t="n"/>
-      <c r="R46" s="59" t="n"/>
-      <c r="S46" s="59" t="n"/>
-      <c r="T46" s="59" t="n"/>
+      <c r="R46" s="95" t="n"/>
+      <c r="S46" s="95" t="n"/>
+      <c r="T46" s="95" t="n"/>
       <c r="U46" s="32" t="n"/>
     </row>
     <row r="47">
@@ -13827,7 +13094,7 @@
       </c>
     </row>
     <row r="4" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B4" s="53" t="n"/>
+      <c r="B4" s="87" t="n"/>
       <c r="C4" s="9" t="inlineStr">
         <is>
           <t>非定常業務</t>
@@ -13861,7 +13128,7 @@
       </c>
     </row>
     <row r="5" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B5" s="53" t="n"/>
+      <c r="B5" s="87" t="n"/>
       <c r="C5" s="9" t="inlineStr">
         <is>
           <t>非定常業務</t>
@@ -13889,7 +13156,7 @@
       </c>
     </row>
     <row r="6" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B6" s="53" t="n"/>
+      <c r="B6" s="87" t="n"/>
       <c r="C6" s="9" t="inlineStr">
         <is>
           <t>非定常業務</t>
@@ -13917,7 +13184,7 @@
       </c>
     </row>
     <row r="7" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B7" s="53" t="n"/>
+      <c r="B7" s="87" t="n"/>
       <c r="C7" s="9" t="inlineStr">
         <is>
           <t>非定常業務</t>
@@ -13945,7 +13212,7 @@
       </c>
     </row>
     <row r="8" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B8" s="53" t="n"/>
+      <c r="B8" s="87" t="n"/>
       <c r="C8" s="9" t="inlineStr">
         <is>
           <t>非定常業務</t>
@@ -13976,7 +13243,7 @@
       <c r="T8" s="1" t="n"/>
     </row>
     <row r="9" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B9" s="53" t="n"/>
+      <c r="B9" s="87" t="n"/>
       <c r="C9" s="9" t="inlineStr">
         <is>
           <t>非定常業務</t>
@@ -14007,7 +13274,7 @@
       <c r="T9" s="1" t="n"/>
     </row>
     <row r="10" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B10" s="53" t="n"/>
+      <c r="B10" s="87" t="n"/>
       <c r="C10" s="9" t="inlineStr">
         <is>
           <t>非定常業務</t>
@@ -14038,7 +13305,7 @@
       <c r="T10" s="1" t="n"/>
     </row>
     <row r="11" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B11" s="53" t="n"/>
+      <c r="B11" s="87" t="n"/>
       <c r="C11" s="9" t="inlineStr">
         <is>
           <t>非定常業務</t>
@@ -14069,7 +13336,7 @@
       <c r="T11" s="1" t="n"/>
     </row>
     <row r="12" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B12" s="53" t="n"/>
+      <c r="B12" s="87" t="n"/>
       <c r="C12" s="9" t="inlineStr">
         <is>
           <t>非定常業務</t>
@@ -14100,7 +13367,7 @@
       <c r="T12" s="1" t="n"/>
     </row>
     <row r="13" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B13" s="53" t="n"/>
+      <c r="B13" s="87" t="n"/>
       <c r="C13" s="9" t="inlineStr">
         <is>
           <t>非定常業務</t>
@@ -14131,7 +13398,7 @@
       <c r="T13" s="1" t="n"/>
     </row>
     <row r="14" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B14" s="54" t="n"/>
+      <c r="B14" s="88" t="n"/>
       <c r="C14" s="9" t="n"/>
       <c r="D14" s="10" t="n"/>
       <c r="E14" s="11" t="n"/>
@@ -14209,11 +13476,11 @@
           <t>掛け数</t>
         </is>
       </c>
-      <c r="S15" s="51" t="n"/>
-      <c r="T15" s="52" t="n"/>
+      <c r="S15" s="89" t="n"/>
+      <c r="T15" s="90" t="n"/>
     </row>
     <row r="16" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B16" s="53" t="n"/>
+      <c r="B16" s="87" t="n"/>
       <c r="C16" s="18" t="inlineStr">
         <is>
           <t>主要外業務</t>
@@ -14265,7 +13532,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="53" t="n"/>
+      <c r="B17" s="87" t="n"/>
       <c r="C17" s="18" t="inlineStr">
         <is>
           <t>主要外業務</t>
@@ -14310,7 +13577,7 @@
       <c r="T17" s="1" t="n"/>
     </row>
     <row r="18">
-      <c r="B18" s="53" t="n"/>
+      <c r="B18" s="87" t="n"/>
       <c r="C18" s="18" t="inlineStr">
         <is>
           <t>主要外業務</t>
@@ -14351,7 +13618,7 @@
       <c r="T18" s="1" t="n"/>
     </row>
     <row r="19">
-      <c r="B19" s="53" t="n"/>
+      <c r="B19" s="87" t="n"/>
       <c r="C19" s="18" t="inlineStr">
         <is>
           <t>主要外業務</t>
@@ -14392,7 +13659,7 @@
       <c r="T19" s="1" t="n"/>
     </row>
     <row r="20">
-      <c r="B20" s="53" t="n"/>
+      <c r="B20" s="87" t="n"/>
       <c r="C20" s="18" t="inlineStr">
         <is>
           <t>主要外業務</t>
@@ -14429,7 +13696,7 @@
       <c r="T20" s="1" t="n"/>
     </row>
     <row r="21">
-      <c r="B21" s="53" t="n"/>
+      <c r="B21" s="87" t="n"/>
       <c r="C21" s="18" t="inlineStr">
         <is>
           <t>主要外業務</t>
@@ -14466,7 +13733,7 @@
       <c r="T21" s="1" t="n"/>
     </row>
     <row r="22">
-      <c r="B22" s="53" t="n"/>
+      <c r="B22" s="87" t="n"/>
       <c r="C22" s="18" t="inlineStr">
         <is>
           <t>主要外業務</t>
@@ -14503,7 +13770,7 @@
       <c r="T22" s="1" t="n"/>
     </row>
     <row r="23">
-      <c r="B23" s="53" t="n"/>
+      <c r="B23" s="87" t="n"/>
       <c r="C23" s="18" t="inlineStr">
         <is>
           <t>主要外業務</t>
@@ -14540,7 +13807,7 @@
       <c r="T23" s="1" t="n"/>
     </row>
     <row r="24">
-      <c r="B24" s="53" t="n"/>
+      <c r="B24" s="87" t="n"/>
       <c r="C24" s="18" t="inlineStr">
         <is>
           <t>主要外業務</t>
@@ -14577,7 +13844,7 @@
       <c r="T24" s="1" t="n"/>
     </row>
     <row r="25">
-      <c r="B25" s="53" t="n"/>
+      <c r="B25" s="87" t="n"/>
       <c r="C25" s="18" t="inlineStr">
         <is>
           <t>主要外業務</t>
@@ -14614,7 +13881,7 @@
       <c r="T25" s="1" t="n"/>
     </row>
     <row r="26">
-      <c r="B26" s="53" t="n"/>
+      <c r="B26" s="87" t="n"/>
       <c r="C26" s="18" t="inlineStr">
         <is>
           <t>主要外業務</t>
@@ -14651,7 +13918,7 @@
       <c r="T26" s="1" t="n"/>
     </row>
     <row r="27">
-      <c r="B27" s="53" t="n"/>
+      <c r="B27" s="87" t="n"/>
       <c r="C27" s="18" t="inlineStr">
         <is>
           <t>主要外業務</t>
@@ -14688,7 +13955,7 @@
       <c r="T27" s="1" t="n"/>
     </row>
     <row r="28" hidden="1">
-      <c r="B28" s="53" t="n"/>
+      <c r="B28" s="87" t="n"/>
       <c r="C28" s="18" t="inlineStr">
         <is>
           <t>主要外業務</t>
@@ -14719,7 +13986,7 @@
       <c r="T28" s="1" t="n"/>
     </row>
     <row r="29" hidden="1">
-      <c r="B29" s="53" t="n"/>
+      <c r="B29" s="87" t="n"/>
       <c r="C29" s="18" t="inlineStr">
         <is>
           <t>主要外業務</t>
@@ -14750,7 +14017,7 @@
       <c r="T29" s="1" t="n"/>
     </row>
     <row r="30" hidden="1">
-      <c r="B30" s="54" t="n"/>
+      <c r="B30" s="88" t="n"/>
       <c r="C30" s="18" t="n"/>
       <c r="D30" s="26" t="n"/>
       <c r="E30" s="16" t="n"/>
@@ -14819,7 +14086,7 @@
       <c r="T31" s="1" t="n"/>
     </row>
     <row r="32">
-      <c r="B32" s="53" t="n"/>
+      <c r="B32" s="87" t="n"/>
       <c r="C32" s="29" t="inlineStr">
         <is>
           <t>主体業務</t>
@@ -14856,7 +14123,7 @@
       <c r="T32" s="1" t="n"/>
     </row>
     <row r="33">
-      <c r="B33" s="53" t="n"/>
+      <c r="B33" s="87" t="n"/>
       <c r="C33" s="29" t="inlineStr">
         <is>
           <t>主体業務</t>
@@ -14893,7 +14160,7 @@
       <c r="T33" s="1" t="n"/>
     </row>
     <row r="34">
-      <c r="B34" s="53" t="n"/>
+      <c r="B34" s="87" t="n"/>
       <c r="C34" s="29" t="inlineStr">
         <is>
           <t>主体業務</t>
@@ -14930,7 +14197,7 @@
       <c r="T34" s="1" t="n"/>
     </row>
     <row r="35">
-      <c r="B35" s="53" t="n"/>
+      <c r="B35" s="87" t="n"/>
       <c r="C35" s="29" t="inlineStr">
         <is>
           <t>主体業務</t>
@@ -14967,7 +14234,7 @@
       <c r="T35" s="1" t="n"/>
     </row>
     <row r="36">
-      <c r="B36" s="53" t="n"/>
+      <c r="B36" s="87" t="n"/>
       <c r="C36" s="29" t="inlineStr">
         <is>
           <t>主体業務</t>
@@ -15004,7 +14271,7 @@
       <c r="T36" s="1" t="n"/>
     </row>
     <row r="37">
-      <c r="B37" s="53" t="n"/>
+      <c r="B37" s="87" t="n"/>
       <c r="C37" s="29" t="inlineStr">
         <is>
           <t>主体業務</t>
@@ -15041,7 +14308,7 @@
       <c r="T37" s="1" t="n"/>
     </row>
     <row r="38">
-      <c r="B38" s="53" t="n"/>
+      <c r="B38" s="87" t="n"/>
       <c r="C38" s="29" t="inlineStr">
         <is>
           <t>主体業務</t>
@@ -15078,7 +14345,7 @@
       <c r="T38" s="1" t="n"/>
     </row>
     <row r="39" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B39" s="53" t="n"/>
+      <c r="B39" s="87" t="n"/>
       <c r="C39" s="29" t="inlineStr">
         <is>
           <t>主体業務</t>
@@ -15115,7 +14382,7 @@
       <c r="T39" s="1" t="n"/>
     </row>
     <row r="40" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B40" s="53" t="n"/>
+      <c r="B40" s="87" t="n"/>
       <c r="C40" s="29" t="inlineStr">
         <is>
           <t>主体業務</t>
@@ -15146,7 +14413,7 @@
       <c r="T40" s="1" t="n"/>
     </row>
     <row r="41" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B41" s="53" t="n"/>
+      <c r="B41" s="87" t="n"/>
       <c r="C41" s="29" t="inlineStr">
         <is>
           <t>主体業務</t>
@@ -15177,7 +14444,7 @@
       <c r="T41" s="1" t="n"/>
     </row>
     <row r="42" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B42" s="53" t="n"/>
+      <c r="B42" s="87" t="n"/>
       <c r="C42" s="29" t="inlineStr">
         <is>
           <t>主体業務</t>
@@ -15208,7 +14475,7 @@
       <c r="T42" s="1" t="n"/>
     </row>
     <row r="43" hidden="1" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B43" s="54" t="n"/>
+      <c r="B43" s="88" t="n"/>
       <c r="C43" s="31" t="n"/>
       <c r="D43" s="27" t="n"/>
       <c r="E43" s="28" t="n"/>
@@ -15242,10 +14509,10 @@
           <t>合計</t>
         </is>
       </c>
-      <c r="D44" s="55" t="n"/>
-      <c r="E44" s="55" t="n"/>
-      <c r="F44" s="55" t="n"/>
-      <c r="G44" s="56" t="n"/>
+      <c r="D44" s="91" t="n"/>
+      <c r="E44" s="91" t="n"/>
+      <c r="F44" s="91" t="n"/>
+      <c r="G44" s="92" t="n"/>
       <c r="H44" s="33">
         <f>SUM(H3:H43)</f>
         <v/>
@@ -15272,10 +14539,10 @@
           <t>実際の勤務時間</t>
         </is>
       </c>
-      <c r="D45" s="57" t="n"/>
-      <c r="E45" s="57" t="n"/>
-      <c r="F45" s="57" t="n"/>
-      <c r="G45" s="58" t="n"/>
+      <c r="D45" s="93" t="n"/>
+      <c r="E45" s="93" t="n"/>
+      <c r="F45" s="93" t="n"/>
+      <c r="G45" s="94" t="n"/>
       <c r="H45" s="50" t="n">
         <v>48.556</v>
       </c>
@@ -15301,15 +14568,15 @@
           <t>比率</t>
         </is>
       </c>
-      <c r="D46" s="57" t="n"/>
-      <c r="E46" s="57" t="n"/>
-      <c r="F46" s="57" t="n"/>
-      <c r="G46" s="58" t="n"/>
+      <c r="D46" s="93" t="n"/>
+      <c r="E46" s="93" t="n"/>
+      <c r="F46" s="93" t="n"/>
+      <c r="G46" s="94" t="n"/>
       <c r="H46" s="37">
         <f>H44/H45</f>
         <v/>
       </c>
-      <c r="I46" s="59" t="n"/>
+      <c r="I46" s="95" t="n"/>
       <c r="J46" s="32" t="n"/>
       <c r="K46" s="32" t="n"/>
       <c r="L46" s="32" t="n"/>
@@ -15318,9 +14585,9 @@
       <c r="O46" s="32" t="n"/>
       <c r="P46" s="32" t="n"/>
       <c r="Q46" s="32" t="n"/>
-      <c r="R46" s="59" t="n"/>
-      <c r="S46" s="59" t="n"/>
-      <c r="T46" s="59" t="n"/>
+      <c r="R46" s="95" t="n"/>
+      <c r="S46" s="95" t="n"/>
+      <c r="T46" s="95" t="n"/>
       <c r="U46" s="32" t="n"/>
     </row>
     <row r="47">
@@ -15358,626 +14625,755 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G24"/>
+  <dimension ref="B2:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="2" ht="24" customHeight="1">
-      <c r="B2" s="60" t="inlineStr">
-        <is>
-          <t>2026年5月12日　業務記録</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="B3" s="61" t="inlineStr">
-        <is>
-          <t>業務分類</t>
-        </is>
-      </c>
-      <c r="C3" s="61" t="inlineStr">
-        <is>
-          <t>業務種別</t>
-        </is>
-      </c>
-      <c r="D3" s="61" t="inlineStr">
+    <row r="2" ht="26" customHeight="1">
+      <c r="B2" s="96" t="inlineStr">
+        <is>
+          <t>2026年5月12日（火）　業務記録</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="B3" s="52" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C3" s="52" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D3" s="52" t="inlineStr">
         <is>
           <t>業務内容</t>
         </is>
       </c>
-      <c r="E3" s="61" t="inlineStr">
+      <c r="E3" s="52" t="inlineStr">
         <is>
           <t>開始</t>
         </is>
       </c>
-      <c r="F3" s="61" t="inlineStr">
+      <c r="F3" s="52" t="inlineStr">
         <is>
           <t>終了</t>
         </is>
       </c>
-      <c r="G3" s="61" t="inlineStr">
+      <c r="G3" s="52" t="inlineStr">
         <is>
           <t>所要時間（分）</t>
         </is>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="B4" s="62" t="inlineStr">
-        <is>
-          <t>付帯業務
-ノンコア業務</t>
-        </is>
-      </c>
-      <c r="C4" s="62" t="inlineStr">
-        <is>
-          <t>主要外業務</t>
-        </is>
-      </c>
-      <c r="D4" s="62" t="inlineStr">
+      <c r="B4" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C4" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D4" s="97" t="inlineStr">
         <is>
           <t>ラジオ体操・各作業場所朝礼</t>
         </is>
       </c>
-      <c r="E4" s="63" t="inlineStr">
+      <c r="E4" s="98" t="inlineStr">
         <is>
           <t>8:00</t>
         </is>
       </c>
-      <c r="F4" s="63" t="inlineStr">
+      <c r="F4" s="98" t="inlineStr">
         <is>
           <t>8:10</t>
         </is>
       </c>
-      <c r="G4" s="63" t="n">
+      <c r="G4" s="98" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="B5" s="64" t="inlineStr">
-        <is>
-          <t>削減可能業務</t>
-        </is>
-      </c>
-      <c r="C5" s="64" t="inlineStr">
-        <is>
-          <t>非定常業務</t>
-        </is>
-      </c>
-      <c r="D5" s="64" t="inlineStr">
-        <is>
-          <t>金峰・川場薄根 打ち合わせ</t>
-        </is>
-      </c>
-      <c r="E5" s="65" t="inlineStr">
+      <c r="B5" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C5" s="58" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D5" s="99" t="inlineStr">
+        <is>
+          <t>金峰・川場薄根 打ち合わせ（現場品物確認）</t>
+        </is>
+      </c>
+      <c r="E5" s="100" t="inlineStr">
         <is>
           <t>8:10</t>
         </is>
       </c>
-      <c r="F5" s="65" t="inlineStr">
+      <c r="F5" s="100" t="inlineStr">
         <is>
           <t>8:25</t>
         </is>
       </c>
-      <c r="G5" s="65" t="n">
+      <c r="G5" s="100" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="B6" s="62" t="inlineStr">
-        <is>
-          <t>付帯業務
-ノンコア業務</t>
-        </is>
-      </c>
-      <c r="C6" s="62" t="inlineStr">
-        <is>
-          <t>主要外業務</t>
-        </is>
-      </c>
-      <c r="D6" s="62" t="inlineStr">
+      <c r="B6" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C6" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D6" s="101" t="inlineStr">
         <is>
           <t>事務作業</t>
         </is>
       </c>
-      <c r="E6" s="63" t="inlineStr">
+      <c r="E6" s="102" t="inlineStr">
         <is>
           <t>8:25</t>
         </is>
       </c>
-      <c r="F6" s="63" t="inlineStr">
+      <c r="F6" s="102" t="inlineStr">
         <is>
           <t>8:46</t>
         </is>
       </c>
-      <c r="G6" s="63" t="n">
+      <c r="G6" s="102" t="n">
         <v>21</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="B7" s="62" t="inlineStr">
-        <is>
-          <t>付帯業務
-ノンコア業務</t>
-        </is>
-      </c>
-      <c r="C7" s="62" t="inlineStr">
-        <is>
-          <t>主要外業務</t>
-        </is>
-      </c>
-      <c r="D7" s="62" t="inlineStr">
+      <c r="B7" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C7" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D7" s="97" t="inlineStr">
         <is>
           <t>笠取工場へ移動</t>
         </is>
       </c>
-      <c r="E7" s="63" t="inlineStr">
+      <c r="E7" s="98" t="inlineStr">
         <is>
           <t>8:46</t>
         </is>
       </c>
-      <c r="F7" s="63" t="inlineStr">
+      <c r="F7" s="98" t="inlineStr">
         <is>
           <t>9:03</t>
         </is>
       </c>
-      <c r="G7" s="63" t="n">
+      <c r="G7" s="98" t="n">
         <v>17</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="B8" s="64" t="inlineStr">
-        <is>
-          <t>削減可能業務</t>
-        </is>
-      </c>
-      <c r="C8" s="64" t="inlineStr">
-        <is>
-          <t>非定常業務</t>
-        </is>
-      </c>
-      <c r="D8" s="64" t="inlineStr">
+      <c r="B8" s="66" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C8" s="66" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D8" s="103" t="inlineStr">
         <is>
           <t>治具の整理</t>
         </is>
       </c>
-      <c r="E8" s="65" t="inlineStr">
+      <c r="E8" s="104" t="inlineStr">
         <is>
           <t>9:03</t>
         </is>
       </c>
-      <c r="F8" s="65" t="inlineStr">
+      <c r="F8" s="104" t="inlineStr">
         <is>
           <t>10:00</t>
         </is>
       </c>
-      <c r="G8" s="65" t="n">
+      <c r="G8" s="104" t="n">
         <v>57</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="B9" s="64" t="inlineStr">
-        <is>
-          <t>削減可能業務</t>
-        </is>
-      </c>
-      <c r="C9" s="64" t="inlineStr">
-        <is>
-          <t>非定常業務</t>
-        </is>
-      </c>
-      <c r="D9" s="64" t="inlineStr">
+      <c r="B9" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C9" s="58" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D9" s="99" t="inlineStr">
         <is>
           <t>ナカモトと打ち合わせ</t>
         </is>
       </c>
-      <c r="E9" s="65" t="inlineStr">
+      <c r="E9" s="100" t="inlineStr">
         <is>
           <t>10:00</t>
         </is>
       </c>
-      <c r="F9" s="65" t="inlineStr">
+      <c r="F9" s="100" t="inlineStr">
         <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="G9" s="65" t="n">
+      <c r="G9" s="100" t="n">
         <v>30</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="B10" s="64" t="inlineStr">
-        <is>
-          <t>削減可能業務</t>
-        </is>
-      </c>
-      <c r="C10" s="64" t="inlineStr">
-        <is>
-          <t>非定常業務</t>
-        </is>
-      </c>
-      <c r="D10" s="64" t="inlineStr">
+      <c r="B10" s="66" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C10" s="66" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D10" s="103" t="inlineStr">
         <is>
           <t>治具の整理（再開）</t>
         </is>
       </c>
-      <c r="E10" s="65" t="inlineStr">
+      <c r="E10" s="104" t="inlineStr">
         <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="F10" s="65" t="inlineStr">
+      <c r="F10" s="104" t="inlineStr">
         <is>
           <t>11:50</t>
         </is>
       </c>
-      <c r="G10" s="65" t="n">
+      <c r="G10" s="104" t="n">
         <v>80</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="B11" s="62" t="inlineStr">
-        <is>
-          <t>付帯業務
-ノンコア業務</t>
-        </is>
-      </c>
-      <c r="C11" s="62" t="inlineStr">
-        <is>
-          <t>主要外業務</t>
-        </is>
-      </c>
-      <c r="D11" s="62" t="inlineStr">
+      <c r="B11" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C11" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D11" s="97" t="inlineStr">
         <is>
           <t>本社工場へ移動</t>
         </is>
       </c>
-      <c r="E11" s="63" t="inlineStr">
+      <c r="E11" s="98" t="inlineStr">
         <is>
           <t>11:50</t>
         </is>
       </c>
-      <c r="F11" s="63" t="inlineStr">
+      <c r="F11" s="98" t="inlineStr">
         <is>
           <t>12:05</t>
         </is>
       </c>
-      <c r="G11" s="63" t="n">
+      <c r="G11" s="98" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="B12" s="62" t="inlineStr">
-        <is>
-          <t>付帯業務
-ノンコア業務</t>
-        </is>
-      </c>
-      <c r="C12" s="62" t="inlineStr">
-        <is>
-          <t>主要外業務</t>
-        </is>
-      </c>
-      <c r="D12" s="62" t="inlineStr">
+      <c r="B12" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C12" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D12" s="97" t="inlineStr">
         <is>
           <t>昼休憩</t>
         </is>
       </c>
-      <c r="E12" s="63" t="inlineStr">
+      <c r="E12" s="98" t="inlineStr">
         <is>
           <t>12:05</t>
         </is>
       </c>
-      <c r="F12" s="63" t="inlineStr">
+      <c r="F12" s="98" t="inlineStr">
         <is>
           <t>12:45</t>
         </is>
       </c>
-      <c r="G12" s="63" t="n">
+      <c r="G12" s="98" t="n">
         <v>40</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="B13" s="62" t="inlineStr">
-        <is>
-          <t>付帯業務
-ノンコア業務</t>
-        </is>
-      </c>
-      <c r="C13" s="62" t="inlineStr">
-        <is>
-          <t>主要外業務</t>
-        </is>
-      </c>
-      <c r="D13" s="62" t="inlineStr">
+      <c r="B13" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C13" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D13" s="97" t="inlineStr">
         <is>
           <t>掃除</t>
         </is>
       </c>
-      <c r="E13" s="63" t="inlineStr">
+      <c r="E13" s="98" t="inlineStr">
         <is>
           <t>12:45</t>
         </is>
       </c>
-      <c r="F13" s="63" t="inlineStr">
+      <c r="F13" s="98" t="inlineStr">
         <is>
           <t>12:50</t>
         </is>
       </c>
-      <c r="G13" s="63" t="n">
+      <c r="G13" s="98" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="B14" s="62" t="inlineStr">
         <is>
-          <t>付帯業務
-ノンコア業務</t>
+          <t>③</t>
         </is>
       </c>
       <c r="C14" s="62" t="inlineStr">
         <is>
-          <t>主要外業務</t>
-        </is>
-      </c>
-      <c r="D14" s="62" t="inlineStr">
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D14" s="105" t="inlineStr">
         <is>
           <t>現場周り</t>
         </is>
       </c>
-      <c r="E14" s="63" t="inlineStr">
+      <c r="E14" s="106" t="inlineStr">
         <is>
           <t>12:50</t>
         </is>
       </c>
-      <c r="F14" s="63" t="inlineStr">
+      <c r="F14" s="106" t="inlineStr">
         <is>
           <t>12:58</t>
         </is>
       </c>
-      <c r="G14" s="63" t="n">
+      <c r="G14" s="106" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="B15" s="62" t="inlineStr">
-        <is>
-          <t>付帯業務
-ノンコア業務</t>
-        </is>
-      </c>
-      <c r="C15" s="62" t="inlineStr">
-        <is>
-          <t>主要外業務</t>
-        </is>
-      </c>
-      <c r="D15" s="62" t="inlineStr">
+      <c r="B15" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C15" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D15" s="101" t="inlineStr">
         <is>
           <t>事務処理（メール・資料）</t>
         </is>
       </c>
-      <c r="E15" s="63" t="inlineStr">
+      <c r="E15" s="102" t="inlineStr">
         <is>
           <t>12:58</t>
         </is>
       </c>
-      <c r="F15" s="63" t="inlineStr">
+      <c r="F15" s="102" t="inlineStr">
         <is>
           <t>13:10</t>
         </is>
       </c>
-      <c r="G15" s="63" t="n">
+      <c r="G15" s="102" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="B16" s="64" t="inlineStr">
-        <is>
-          <t>削減可能業務</t>
-        </is>
-      </c>
-      <c r="C16" s="64" t="inlineStr">
-        <is>
-          <t>非定常業務</t>
-        </is>
-      </c>
-      <c r="D16" s="64" t="inlineStr">
+      <c r="B16" s="54" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C16" s="54" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D16" s="107" t="inlineStr">
         <is>
           <t>京都銀行来社 対応</t>
         </is>
       </c>
-      <c r="E16" s="65" t="inlineStr">
+      <c r="E16" s="108" t="inlineStr">
         <is>
           <t>13:10</t>
         </is>
       </c>
-      <c r="F16" s="65" t="inlineStr">
+      <c r="F16" s="108" t="inlineStr">
         <is>
           <t>15:00</t>
         </is>
       </c>
-      <c r="G16" s="65" t="n">
+      <c r="G16" s="108" t="n">
         <v>110</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="B17" s="62" t="inlineStr">
-        <is>
-          <t>付帯業務
-ノンコア業務</t>
-        </is>
-      </c>
-      <c r="C17" s="62" t="inlineStr">
-        <is>
-          <t>主要外業務</t>
-        </is>
-      </c>
-      <c r="D17" s="62" t="inlineStr">
+      <c r="B17" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C17" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D17" s="97" t="inlineStr">
         <is>
           <t>休憩</t>
         </is>
       </c>
-      <c r="E17" s="63" t="inlineStr">
+      <c r="E17" s="98" t="inlineStr">
         <is>
           <t>15:00</t>
         </is>
       </c>
-      <c r="F17" s="63" t="inlineStr">
+      <c r="F17" s="98" t="inlineStr">
         <is>
           <t>15:10</t>
         </is>
       </c>
-      <c r="G17" s="63" t="n">
+      <c r="G17" s="98" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="B18" s="62" t="inlineStr">
-        <is>
-          <t>付帯業務
-ノンコア業務</t>
-        </is>
-      </c>
-      <c r="C18" s="62" t="inlineStr">
-        <is>
-          <t>主要外業務</t>
-        </is>
-      </c>
-      <c r="D18" s="62" t="inlineStr">
+      <c r="B18" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C18" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D18" s="101" t="inlineStr">
         <is>
           <t>事務作業</t>
         </is>
       </c>
-      <c r="E18" s="63" t="inlineStr">
+      <c r="E18" s="102" t="inlineStr">
         <is>
           <t>15:10</t>
         </is>
       </c>
-      <c r="F18" s="63" t="inlineStr">
+      <c r="F18" s="102" t="inlineStr">
         <is>
           <t>15:50</t>
         </is>
       </c>
-      <c r="G18" s="63" t="n">
+      <c r="G18" s="102" t="n">
         <v>40</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="B19" s="62" t="inlineStr">
         <is>
-          <t>付帯業務
-ノンコア業務</t>
+          <t>③</t>
         </is>
       </c>
       <c r="C19" s="62" t="inlineStr">
         <is>
-          <t>主要外業務</t>
-        </is>
-      </c>
-      <c r="D19" s="62" t="inlineStr">
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D19" s="105" t="inlineStr">
         <is>
           <t>現場周り</t>
         </is>
       </c>
-      <c r="E19" s="63" t="inlineStr">
+      <c r="E19" s="106" t="inlineStr">
         <is>
           <t>15:50</t>
         </is>
       </c>
-      <c r="F19" s="63" t="inlineStr">
+      <c r="F19" s="106" t="inlineStr">
         <is>
           <t>16:19</t>
         </is>
       </c>
-      <c r="G19" s="63" t="n">
+      <c r="G19" s="106" t="n">
         <v>29</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="B20" s="62" t="inlineStr">
-        <is>
-          <t>付帯業務
-ノンコア業務</t>
-        </is>
-      </c>
-      <c r="C20" s="62" t="inlineStr">
-        <is>
-          <t>主要外業務</t>
-        </is>
-      </c>
-      <c r="D20" s="62" t="inlineStr">
-        <is>
-          <t>事務処理（メール・資料・報告書）</t>
-        </is>
-      </c>
-      <c r="E20" s="63" t="inlineStr">
+      <c r="B20" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C20" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D20" s="101" t="inlineStr">
+        <is>
+          <t>事務処理（メール・資料・報告書作成）</t>
+        </is>
+      </c>
+      <c r="E20" s="102" t="inlineStr">
         <is>
           <t>16:19</t>
         </is>
       </c>
-      <c r="F20" s="63" t="inlineStr">
+      <c r="F20" s="102" t="inlineStr">
         <is>
           <t>18:08</t>
         </is>
       </c>
-      <c r="G20" s="63" t="n">
+      <c r="G20" s="102" t="n">
         <v>109</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="B22" s="66" t="n"/>
-      <c r="C22" s="67" t="inlineStr">
-        <is>
-          <t>削減可能業務　合計</t>
-        </is>
-      </c>
-      <c r="D22" s="66" t="n"/>
-      <c r="E22" s="66" t="n"/>
-      <c r="F22" s="66" t="n"/>
-      <c r="G22" s="67" t="n">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="B23" s="68" t="n"/>
-      <c r="C23" s="69" t="inlineStr">
-        <is>
-          <t>付帯業務ノンコア業務　合計</t>
-        </is>
-      </c>
-      <c r="D23" s="68" t="n"/>
-      <c r="E23" s="68" t="n"/>
-      <c r="F23" s="68" t="n"/>
-      <c r="G23" s="69" t="n">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="B24" s="70" t="n"/>
-      <c r="C24" s="71" t="inlineStr">
-        <is>
-          <t>総合計</t>
-        </is>
-      </c>
-      <c r="D24" s="70" t="n"/>
-      <c r="E24" s="70" t="n"/>
-      <c r="F24" s="70" t="n"/>
-      <c r="G24" s="71" t="n">
+      <c r="B22" s="52" t="inlineStr">
+        <is>
+          <t>【カテゴリ別集計】</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="52" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C23" s="52" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D23" s="52" t="inlineStr">
+        <is>
+          <t>合計（分）</t>
+        </is>
+      </c>
+      <c r="E23" s="52" t="inlineStr">
+        <is>
+          <t>合計（時間）</t>
+        </is>
+      </c>
+      <c r="F23" s="52" t="inlineStr">
+        <is>
+          <t>割合（%）</t>
+        </is>
+      </c>
+      <c r="G23" s="53" t="n"/>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="B24" s="54" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C24" s="55" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D24" s="108" t="n">
+        <v>110</v>
+      </c>
+      <c r="E24" s="108" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F24" s="108" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="G24" s="57" t="n"/>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="B25" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C25" s="59" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D25" s="100" t="n">
+        <v>45</v>
+      </c>
+      <c r="E25" s="100" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F25" s="100" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="G25" s="61" t="n"/>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="B26" s="62" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C26" s="63" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D26" s="106" t="n">
+        <v>37</v>
+      </c>
+      <c r="E26" s="106" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F26" s="106" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="G26" s="65" t="n"/>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="B27" s="66" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C27" s="67" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D27" s="104" t="n">
+        <v>137</v>
+      </c>
+      <c r="E27" s="104" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="F27" s="104" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="G27" s="69" t="n"/>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="B28" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C28" s="71" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D28" s="102" t="n">
+        <v>182</v>
+      </c>
+      <c r="E28" s="102" t="n">
+        <v>3</v>
+      </c>
+      <c r="F28" s="102" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="G28" s="73" t="n"/>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="B29" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C29" s="75" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D29" s="98" t="n">
+        <v>97</v>
+      </c>
+      <c r="E29" s="98" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="F29" s="98" t="n">
+        <v>16</v>
+      </c>
+      <c r="G29" s="77" t="n"/>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="B30" s="86" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="C30" s="86" t="inlineStr"/>
+      <c r="D30" s="86" t="n">
         <v>608</v>
       </c>
+      <c r="E30" s="86" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="F30" s="86" t="n">
+        <v>100</v>
+      </c>
+      <c r="G30" s="109" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="C22:F22"/>
+  <mergeCells count="2">
+    <mergeCell ref="B22:G22"/>
     <mergeCell ref="B2:G2"/>
-    <mergeCell ref="C24:F24"/>
-    <mergeCell ref="C23:F23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add daily task record for 2026-05-13
Notable: 64% office/admin work (estimate creation, email),
emergency rainwater flooding response (42min), no external meetings.

https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録_2026-05-12.xlsx
+++ b/業務記録_2026-05-12.xlsx
@@ -10,14 +10,15 @@
     <sheet name="１日（例）" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="1週間（例）" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="2026-05-12" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="2026-05-13" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId5"/>
     <externalReference r:id="rId6"/>
     <externalReference r:id="rId7"/>
     <externalReference r:id="rId8"/>
     <externalReference r:id="rId9"/>
     <externalReference r:id="rId10"/>
+    <externalReference r:id="rId11"/>
   </externalReferences>
   <definedNames>
     <definedName name="_13月">#REF!</definedName>
@@ -587,7 +588,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="32">
+  <borders count="41">
     <border>
       <left/>
       <right/>
@@ -961,11 +962,74 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="110">
+  <cellXfs count="116">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -1244,6 +1308,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -1423,7 +1493,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t/>
+                    <a:t>None</a:t>
                   </a:r>
                   <a:endParaRPr lang="ja-JP"/>
                 </a:p>
@@ -1460,7 +1530,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t/>
+                    <a:t>None</a:t>
                   </a:r>
                   <a:endParaRPr lang="ja-JP"/>
                 </a:p>
@@ -1497,7 +1567,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t/>
+                    <a:t>None</a:t>
                   </a:r>
                   <a:endParaRPr lang="ja-JP"/>
                 </a:p>
@@ -1534,7 +1604,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="ja-JP"/>
               </a:p>
@@ -2055,7 +2125,7 @@
             <a:defRPr/>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="ja-JP"/>
         </a:p>
@@ -2170,7 +2240,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t/>
+                    <a:t>None</a:t>
                   </a:r>
                   <a:endParaRPr lang="ja-JP"/>
                 </a:p>
@@ -2207,7 +2277,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t/>
+                    <a:t>None</a:t>
                   </a:r>
                   <a:endParaRPr lang="ja-JP"/>
                 </a:p>
@@ -2244,7 +2314,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t/>
+                    <a:t>None</a:t>
                   </a:r>
                   <a:endParaRPr lang="ja-JP"/>
                 </a:p>
@@ -2281,7 +2351,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="ja-JP"/>
               </a:p>
@@ -2617,7 +2687,7 @@
             <a:defRPr/>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="ja-JP"/>
         </a:p>
@@ -2732,7 +2802,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t/>
+                    <a:t>None</a:t>
                   </a:r>
                   <a:endParaRPr lang="ja-JP"/>
                 </a:p>
@@ -2769,7 +2839,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t/>
+                    <a:t>None</a:t>
                   </a:r>
                   <a:endParaRPr lang="ja-JP"/>
                 </a:p>
@@ -2806,7 +2876,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t/>
+                    <a:t>None</a:t>
                   </a:r>
                   <a:endParaRPr lang="ja-JP"/>
                 </a:p>
@@ -2843,7 +2913,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="ja-JP"/>
               </a:p>
@@ -3359,7 +3429,7 @@
             <a:defRPr/>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="ja-JP"/>
         </a:p>
@@ -10879,7 +10949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G45"/>
+  <dimension ref="B2:T46"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.875" defaultRowHeight="18.75"/>
   <cols>
     <col width="13.375" customWidth="1" min="1" max="1"/>
@@ -10902,21 +10972,25 @@
           <t>取締役工場長　業務記録フォーマット</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="19.5" customHeight="1" thickBot="1"/>
+      <c r="C2" s="110" t="n"/>
+      <c r="D2" s="110" t="n"/>
+      <c r="E2" s="110" t="n"/>
+      <c r="F2" s="110" t="n"/>
+      <c r="G2" s="111" t="n"/>
+    </row>
+    <row r="3" ht="19.5" customHeight="1" thickBot="1">
+      <c r="B3" s="112" t="n"/>
+    </row>
     <row r="4" ht="20" customHeight="1" thickBot="1">
-      <c r="B4" s="52" t="inlineStr">
-        <is>
-          <t>【カテゴリ定義】</t>
-        </is>
-      </c>
+      <c r="B4" s="113" t="n"/>
+      <c r="C4" s="110" t="n"/>
+      <c r="D4" s="110" t="n"/>
+      <c r="E4" s="110" t="n"/>
+      <c r="F4" s="110" t="n"/>
+      <c r="G4" s="111" t="n"/>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="B5" s="52" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
+      <c r="B5" s="113" t="n"/>
       <c r="C5" s="52" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
@@ -10932,11 +11006,7 @@
       <c r="G5" s="53" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="54" t="inlineStr">
-        <is>
-          <t>①</t>
-        </is>
-      </c>
+      <c r="B6" s="113" t="n"/>
       <c r="C6" s="55" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
@@ -10948,15 +11018,11 @@
         </is>
       </c>
       <c r="E6" s="57" t="n"/>
-      <c r="F6" s="57" t="n"/>
-      <c r="G6" s="57" t="n"/>
+      <c r="F6" s="110" t="n"/>
+      <c r="G6" s="111" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="58" t="inlineStr">
-        <is>
-          <t>②</t>
-        </is>
-      </c>
+      <c r="B7" s="113" t="n"/>
       <c r="C7" s="59" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
@@ -10968,15 +11034,11 @@
         </is>
       </c>
       <c r="E7" s="61" t="n"/>
-      <c r="F7" s="61" t="n"/>
-      <c r="G7" s="61" t="n"/>
+      <c r="F7" s="110" t="n"/>
+      <c r="G7" s="111" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="62" t="inlineStr">
-        <is>
-          <t>③</t>
-        </is>
-      </c>
+      <c r="B8" s="113" t="n"/>
       <c r="C8" s="63" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
@@ -10988,15 +11050,11 @@
         </is>
       </c>
       <c r="E8" s="65" t="n"/>
-      <c r="F8" s="65" t="n"/>
-      <c r="G8" s="65" t="n"/>
+      <c r="F8" s="110" t="n"/>
+      <c r="G8" s="111" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="66" t="inlineStr">
-        <is>
-          <t>④</t>
-        </is>
-      </c>
+      <c r="B9" s="113" t="n"/>
       <c r="C9" s="67" t="inlineStr">
         <is>
           <t>現場直接作業</t>
@@ -11008,15 +11066,11 @@
         </is>
       </c>
       <c r="E9" s="69" t="n"/>
-      <c r="F9" s="69" t="n"/>
-      <c r="G9" s="69" t="n"/>
+      <c r="F9" s="110" t="n"/>
+      <c r="G9" s="111" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="70" t="inlineStr">
-        <is>
-          <t>⑤</t>
-        </is>
-      </c>
+      <c r="B10" s="113" t="n"/>
       <c r="C10" s="71" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
@@ -11028,15 +11082,11 @@
         </is>
       </c>
       <c r="E10" s="73" t="n"/>
-      <c r="F10" s="73" t="n"/>
-      <c r="G10" s="73" t="n"/>
+      <c r="F10" s="110" t="n"/>
+      <c r="G10" s="111" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="74" t="inlineStr">
-        <is>
-          <t>⑥</t>
-        </is>
-      </c>
+      <c r="B11" s="113" t="n"/>
       <c r="C11" s="75" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
@@ -11048,15 +11098,22 @@
         </is>
       </c>
       <c r="E11" s="77" t="n"/>
-      <c r="F11" s="77" t="n"/>
-      <c r="G11" s="77" t="n"/>
+      <c r="F11" s="110" t="n"/>
+      <c r="G11" s="111" t="n"/>
+    </row>
+    <row r="12">
+      <c r="B12" s="113" t="n"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="113" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="B14" s="52" t="inlineStr">
-        <is>
-          <t>【日次入力テンプレート】　　日付：</t>
-        </is>
-      </c>
+      <c r="B14" s="112" t="n"/>
+      <c r="C14" s="110" t="n"/>
+      <c r="D14" s="110" t="n"/>
+      <c r="E14" s="110" t="n"/>
+      <c r="F14" s="110" t="n"/>
+      <c r="G14" s="111" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="B15" s="52" t="inlineStr">
@@ -11091,7 +11148,7 @@
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="B16" s="78" t="n"/>
+      <c r="B16" s="114" t="n"/>
       <c r="C16" s="78" t="n"/>
       <c r="D16" s="78" t="n"/>
       <c r="E16" s="78" t="n"/>
@@ -11099,7 +11156,7 @@
       <c r="G16" s="78" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="B17" s="79" t="n"/>
+      <c r="B17" s="114" t="n"/>
       <c r="C17" s="79" t="n"/>
       <c r="D17" s="79" t="n"/>
       <c r="E17" s="79" t="n"/>
@@ -11107,7 +11164,7 @@
       <c r="G17" s="79" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="B18" s="78" t="n"/>
+      <c r="B18" s="114" t="n"/>
       <c r="C18" s="78" t="n"/>
       <c r="D18" s="78" t="n"/>
       <c r="E18" s="78" t="n"/>
@@ -11115,7 +11172,7 @@
       <c r="G18" s="78" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="B19" s="79" t="n"/>
+      <c r="B19" s="114" t="n"/>
       <c r="C19" s="79" t="n"/>
       <c r="D19" s="79" t="n"/>
       <c r="E19" s="79" t="n"/>
@@ -11123,7 +11180,7 @@
       <c r="G19" s="79" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="B20" s="78" t="n"/>
+      <c r="B20" s="114" t="n"/>
       <c r="C20" s="78" t="n"/>
       <c r="D20" s="78" t="n"/>
       <c r="E20" s="78" t="n"/>
@@ -11131,7 +11188,7 @@
       <c r="G20" s="78" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="B21" s="79" t="n"/>
+      <c r="B21" s="114" t="n"/>
       <c r="C21" s="79" t="n"/>
       <c r="D21" s="79" t="n"/>
       <c r="E21" s="79" t="n"/>
@@ -11139,7 +11196,7 @@
       <c r="G21" s="79" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="B22" s="78" t="n"/>
+      <c r="B22" s="114" t="n"/>
       <c r="C22" s="78" t="n"/>
       <c r="D22" s="78" t="n"/>
       <c r="E22" s="78" t="n"/>
@@ -11147,7 +11204,7 @@
       <c r="G22" s="78" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="B23" s="79" t="n"/>
+      <c r="B23" s="114" t="n"/>
       <c r="C23" s="79" t="n"/>
       <c r="D23" s="79" t="n"/>
       <c r="E23" s="79" t="n"/>
@@ -11155,7 +11212,7 @@
       <c r="G23" s="79" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="B24" s="78" t="n"/>
+      <c r="B24" s="114" t="n"/>
       <c r="C24" s="78" t="n"/>
       <c r="D24" s="78" t="n"/>
       <c r="E24" s="78" t="n"/>
@@ -11163,7 +11220,7 @@
       <c r="G24" s="78" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="B25" s="79" t="n"/>
+      <c r="B25" s="114" t="n"/>
       <c r="C25" s="79" t="n"/>
       <c r="D25" s="79" t="n"/>
       <c r="E25" s="79" t="n"/>
@@ -11171,7 +11228,7 @@
       <c r="G25" s="79" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="B26" s="78" t="n"/>
+      <c r="B26" s="114" t="n"/>
       <c r="C26" s="78" t="n"/>
       <c r="D26" s="78" t="n"/>
       <c r="E26" s="78" t="n"/>
@@ -11179,7 +11236,7 @@
       <c r="G26" s="78" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="B27" s="79" t="n"/>
+      <c r="B27" s="114" t="n"/>
       <c r="C27" s="79" t="n"/>
       <c r="D27" s="79" t="n"/>
       <c r="E27" s="79" t="n"/>
@@ -11187,7 +11244,7 @@
       <c r="G27" s="79" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="B28" s="78" t="n"/>
+      <c r="B28" s="114" t="n"/>
       <c r="C28" s="78" t="n"/>
       <c r="D28" s="78" t="n"/>
       <c r="E28" s="78" t="n"/>
@@ -11195,7 +11252,7 @@
       <c r="G28" s="78" t="n"/>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="B29" s="79" t="n"/>
+      <c r="B29" s="114" t="n"/>
       <c r="C29" s="79" t="n"/>
       <c r="D29" s="79" t="n"/>
       <c r="E29" s="79" t="n"/>
@@ -11203,7 +11260,7 @@
       <c r="G29" s="79" t="n"/>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="B30" s="78" t="n"/>
+      <c r="B30" s="115" t="n"/>
       <c r="C30" s="78" t="n"/>
       <c r="D30" s="78" t="n"/>
       <c r="E30" s="78" t="n"/>
@@ -11219,7 +11276,7 @@
       <c r="G31" s="79" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="B32" s="78" t="n"/>
+      <c r="B32" s="114" t="n"/>
       <c r="C32" s="78" t="n"/>
       <c r="D32" s="78" t="n"/>
       <c r="E32" s="78" t="n"/>
@@ -11227,7 +11284,7 @@
       <c r="G32" s="78" t="n"/>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="B33" s="79" t="n"/>
+      <c r="B33" s="114" t="n"/>
       <c r="C33" s="79" t="n"/>
       <c r="D33" s="79" t="n"/>
       <c r="E33" s="79" t="n"/>
@@ -11235,7 +11292,7 @@
       <c r="G33" s="79" t="n"/>
     </row>
     <row r="34" ht="18" customHeight="1">
-      <c r="B34" s="78" t="n"/>
+      <c r="B34" s="114" t="n"/>
       <c r="C34" s="78" t="n"/>
       <c r="D34" s="78" t="n"/>
       <c r="E34" s="78" t="n"/>
@@ -11243,26 +11300,22 @@
       <c r="G34" s="78" t="n"/>
     </row>
     <row r="35" ht="18" customHeight="1">
-      <c r="B35" s="79" t="n"/>
+      <c r="B35" s="114" t="n"/>
       <c r="C35" s="79" t="n"/>
       <c r="D35" s="79" t="n"/>
       <c r="E35" s="79" t="n"/>
       <c r="F35" s="79" t="n"/>
       <c r="G35" s="79" t="n"/>
     </row>
+    <row r="36">
+      <c r="B36" s="114" t="n"/>
+    </row>
     <row r="37" ht="20" customHeight="1">
-      <c r="B37" s="52" t="inlineStr">
-        <is>
-          <t>【カテゴリ別集計】</t>
-        </is>
-      </c>
+      <c r="B37" s="114" t="n"/>
+      <c r="G37" s="113" t="n"/>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="B38" s="52" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
+      <c r="B38" s="114" t="n"/>
       <c r="C38" s="52" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
@@ -11290,11 +11343,7 @@
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="B39" s="54" t="inlineStr">
-        <is>
-          <t>①</t>
-        </is>
-      </c>
+      <c r="B39" s="114" t="n"/>
       <c r="C39" s="80" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
@@ -11306,11 +11355,7 @@
       <c r="G39" s="57" t="n"/>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="B40" s="58" t="inlineStr">
-        <is>
-          <t>②</t>
-        </is>
-      </c>
+      <c r="B40" s="114" t="n"/>
       <c r="C40" s="81" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
@@ -11322,11 +11367,7 @@
       <c r="G40" s="61" t="n"/>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="B41" s="62" t="inlineStr">
-        <is>
-          <t>③</t>
-        </is>
-      </c>
+      <c r="B41" s="114" t="n"/>
       <c r="C41" s="82" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
@@ -11338,11 +11379,7 @@
       <c r="G41" s="65" t="n"/>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="B42" s="66" t="inlineStr">
-        <is>
-          <t>④</t>
-        </is>
-      </c>
+      <c r="B42" s="114" t="n"/>
       <c r="C42" s="83" t="inlineStr">
         <is>
           <t>現場直接作業</t>
@@ -11354,11 +11391,7 @@
       <c r="G42" s="69" t="n"/>
     </row>
     <row r="43" ht="18" customHeight="1" thickBot="1">
-      <c r="B43" s="70" t="inlineStr">
-        <is>
-          <t>⑤</t>
-        </is>
-      </c>
+      <c r="B43" s="115" t="n"/>
       <c r="C43" s="84" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
@@ -11380,10 +11413,10 @@
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D44" s="77" t="n"/>
-      <c r="E44" s="77" t="n"/>
-      <c r="F44" s="77" t="n"/>
-      <c r="G44" s="77" t="n"/>
+      <c r="D44" s="110" t="n"/>
+      <c r="E44" s="110" t="n"/>
+      <c r="F44" s="110" t="n"/>
+      <c r="G44" s="111" t="n"/>
     </row>
     <row r="45" ht="20" customHeight="1">
       <c r="B45" s="86" t="inlineStr">
@@ -11392,10 +11425,10 @@
         </is>
       </c>
       <c r="C45" s="86" t="n"/>
-      <c r="D45" s="86" t="n"/>
-      <c r="E45" s="86" t="n"/>
-      <c r="F45" s="86" t="n"/>
-      <c r="G45" s="86" t="n"/>
+      <c r="D45" s="110" t="n"/>
+      <c r="E45" s="110" t="n"/>
+      <c r="F45" s="110" t="n"/>
+      <c r="G45" s="111" t="n"/>
     </row>
     <row r="46" ht="24" customHeight="1"/>
   </sheetData>
@@ -11403,8 +11436,8 @@
     <mergeCell ref="B31:B43"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="E10:G10"/>
+    <mergeCell ref="E11:G11"/>
     <mergeCell ref="R3:T3"/>
-    <mergeCell ref="E11:G11"/>
     <mergeCell ref="C46:G46"/>
     <mergeCell ref="B14:G14"/>
     <mergeCell ref="B37:G37"/>
@@ -14642,6 +14675,11 @@
           <t>2026年5月12日（火）　業務記録</t>
         </is>
       </c>
+      <c r="C2" s="110" t="n"/>
+      <c r="D2" s="110" t="n"/>
+      <c r="E2" s="110" t="n"/>
+      <c r="F2" s="110" t="n"/>
+      <c r="G2" s="111" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="B3" s="52" t="inlineStr">
@@ -15191,6 +15229,11 @@
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
+      <c r="C22" s="110" t="n"/>
+      <c r="D22" s="110" t="n"/>
+      <c r="E22" s="110" t="n"/>
+      <c r="F22" s="110" t="n"/>
+      <c r="G22" s="111" t="n"/>
     </row>
     <row r="23">
       <c r="B23" s="52" t="inlineStr">
@@ -15377,4 +15420,794 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:G31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="26" customHeight="1">
+      <c r="B2" s="96" t="inlineStr">
+        <is>
+          <t>2026年5月13日（水）　業務記録</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="B3" s="52" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C3" s="52" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D3" s="52" t="inlineStr">
+        <is>
+          <t>業務内容</t>
+        </is>
+      </c>
+      <c r="E3" s="52" t="inlineStr">
+        <is>
+          <t>開始</t>
+        </is>
+      </c>
+      <c r="F3" s="52" t="inlineStr">
+        <is>
+          <t>終了</t>
+        </is>
+      </c>
+      <c r="G3" s="52" t="inlineStr">
+        <is>
+          <t>所要時間（分）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="B4" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C4" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D4" s="101" t="inlineStr">
+        <is>
+          <t>メールチェック・返信・事務作業</t>
+        </is>
+      </c>
+      <c r="E4" s="102" t="inlineStr">
+        <is>
+          <t>7:37</t>
+        </is>
+      </c>
+      <c r="F4" s="102" t="inlineStr">
+        <is>
+          <t>7:44</t>
+        </is>
+      </c>
+      <c r="G4" s="102" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="B5" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C5" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D5" s="97" t="inlineStr">
+        <is>
+          <t>休憩</t>
+        </is>
+      </c>
+      <c r="E5" s="98" t="inlineStr">
+        <is>
+          <t>7:44</t>
+        </is>
+      </c>
+      <c r="F5" s="98" t="inlineStr">
+        <is>
+          <t>8:00</t>
+        </is>
+      </c>
+      <c r="G5" s="98" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="B6" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C6" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D6" s="97" t="inlineStr">
+        <is>
+          <t>ラジオ体操</t>
+        </is>
+      </c>
+      <c r="E6" s="98" t="inlineStr">
+        <is>
+          <t>8:00</t>
+        </is>
+      </c>
+      <c r="F6" s="98" t="inlineStr">
+        <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="G6" s="98" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="B7" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C7" s="58" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D7" s="99" t="inlineStr">
+        <is>
+          <t>鉄心工場・コイル工場 朝礼参加</t>
+        </is>
+      </c>
+      <c r="E7" s="100" t="inlineStr">
+        <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="F7" s="100" t="inlineStr">
+        <is>
+          <t>8:07</t>
+        </is>
+      </c>
+      <c r="G7" s="100" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="B8" s="62" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C8" s="62" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D8" s="105" t="inlineStr">
+        <is>
+          <t>現場周り（挨拶・品物確認）</t>
+        </is>
+      </c>
+      <c r="E8" s="106" t="inlineStr">
+        <is>
+          <t>8:08</t>
+        </is>
+      </c>
+      <c r="F8" s="106" t="inlineStr">
+        <is>
+          <t>8:16</t>
+        </is>
+      </c>
+      <c r="G8" s="106" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="B9" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C9" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D9" s="97" t="inlineStr">
+        <is>
+          <t>トイレ</t>
+        </is>
+      </c>
+      <c r="E9" s="98" t="inlineStr">
+        <is>
+          <t>8:16</t>
+        </is>
+      </c>
+      <c r="F9" s="98" t="inlineStr">
+        <is>
+          <t>8:17</t>
+        </is>
+      </c>
+      <c r="G9" s="98" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="B10" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C10" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D10" s="101" t="inlineStr">
+        <is>
+          <t>事務作業（返信・報告書確認・見積書作成・電話対応・打合含む）</t>
+        </is>
+      </c>
+      <c r="E10" s="102" t="inlineStr">
+        <is>
+          <t>8:17</t>
+        </is>
+      </c>
+      <c r="F10" s="102" t="inlineStr">
+        <is>
+          <t>10:02</t>
+        </is>
+      </c>
+      <c r="G10" s="102" t="n">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="B11" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C11" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D11" s="97" t="inlineStr">
+        <is>
+          <t>休憩</t>
+        </is>
+      </c>
+      <c r="E11" s="98" t="inlineStr">
+        <is>
+          <t>10:02</t>
+        </is>
+      </c>
+      <c r="F11" s="98" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="G11" s="98" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="B12" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C12" s="58" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D12" s="99" t="inlineStr">
+        <is>
+          <t>現場ミニ製造会議（品物確認）</t>
+        </is>
+      </c>
+      <c r="E12" s="100" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="F12" s="100" t="inlineStr">
+        <is>
+          <t>10:48</t>
+        </is>
+      </c>
+      <c r="G12" s="100" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="B13" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C13" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D13" s="101" t="inlineStr">
+        <is>
+          <t>事務作業（見積書作成・メール返答・見積回答）</t>
+        </is>
+      </c>
+      <c r="E13" s="102" t="inlineStr">
+        <is>
+          <t>10:48</t>
+        </is>
+      </c>
+      <c r="F13" s="102" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="G13" s="102" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="B14" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C14" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D14" s="97" t="inlineStr">
+        <is>
+          <t>昼休憩</t>
+        </is>
+      </c>
+      <c r="E14" s="98" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="F14" s="98" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="G14" s="98" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="B15" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C15" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D15" s="97" t="inlineStr">
+        <is>
+          <t>掃除</t>
+        </is>
+      </c>
+      <c r="E15" s="98" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="F15" s="98" t="inlineStr">
+        <is>
+          <t>12:56</t>
+        </is>
+      </c>
+      <c r="G15" s="98" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="B16" s="62" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C16" s="62" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D16" s="105" t="inlineStr">
+        <is>
+          <t>現場周り</t>
+        </is>
+      </c>
+      <c r="E16" s="106" t="inlineStr">
+        <is>
+          <t>12:56</t>
+        </is>
+      </c>
+      <c r="F16" s="106" t="inlineStr">
+        <is>
+          <t>13:11</t>
+        </is>
+      </c>
+      <c r="G16" s="106" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="B17" s="66" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C17" s="66" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D17" s="103" t="inlineStr">
+        <is>
+          <t>雨水浸水対応（緊急・ゲリラ）</t>
+        </is>
+      </c>
+      <c r="E17" s="104" t="inlineStr">
+        <is>
+          <t>13:11</t>
+        </is>
+      </c>
+      <c r="F17" s="104" t="inlineStr">
+        <is>
+          <t>13:53</t>
+        </is>
+      </c>
+      <c r="G17" s="104" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="B18" s="62" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C18" s="62" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D18" s="105" t="inlineStr">
+        <is>
+          <t>現場確認・見回り</t>
+        </is>
+      </c>
+      <c r="E18" s="106" t="inlineStr">
+        <is>
+          <t>13:53</t>
+        </is>
+      </c>
+      <c r="F18" s="106" t="inlineStr">
+        <is>
+          <t>14:04</t>
+        </is>
+      </c>
+      <c r="G18" s="106" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="B19" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C19" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D19" s="101" t="inlineStr">
+        <is>
+          <t>事務作業（メールチェック・見積・返信）</t>
+        </is>
+      </c>
+      <c r="E19" s="102" t="inlineStr">
+        <is>
+          <t>14:04</t>
+        </is>
+      </c>
+      <c r="F19" s="102" t="inlineStr">
+        <is>
+          <t>16:25</t>
+        </is>
+      </c>
+      <c r="G19" s="102" t="n">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="B20" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C20" s="58" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D20" s="99" t="inlineStr">
+        <is>
+          <t>フォークリフト法定点検 関係者打ち合わせ</t>
+        </is>
+      </c>
+      <c r="E20" s="100" t="inlineStr">
+        <is>
+          <t>16:25</t>
+        </is>
+      </c>
+      <c r="F20" s="100" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="G20" s="100" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="B21" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C21" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D21" s="101" t="inlineStr">
+        <is>
+          <t>事務作業（再開）</t>
+        </is>
+      </c>
+      <c r="E21" s="102" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="F21" s="102" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="G21" s="102" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="B23" s="52" t="inlineStr">
+        <is>
+          <t>【カテゴリ別集計】</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="52" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C24" s="52" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D24" s="52" t="inlineStr">
+        <is>
+          <t>合計（分）</t>
+        </is>
+      </c>
+      <c r="E24" s="52" t="inlineStr">
+        <is>
+          <t>合計（時間）</t>
+        </is>
+      </c>
+      <c r="F24" s="52" t="inlineStr">
+        <is>
+          <t>割合（%）</t>
+        </is>
+      </c>
+      <c r="G24" s="53" t="n"/>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="B25" s="54" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C25" s="55" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D25" s="108" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="108" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="108" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="57" t="n"/>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="B26" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C26" s="59" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D26" s="100" t="n">
+        <v>62</v>
+      </c>
+      <c r="E26" s="100" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="100" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="G26" s="61" t="n"/>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="B27" s="62" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C27" s="63" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D27" s="106" t="n">
+        <v>34</v>
+      </c>
+      <c r="E27" s="106" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F27" s="106" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="G27" s="65" t="n"/>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="B28" s="66" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C28" s="67" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D28" s="104" t="n">
+        <v>42</v>
+      </c>
+      <c r="E28" s="104" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F28" s="104" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="G28" s="69" t="n"/>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="B29" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C29" s="71" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D29" s="102" t="n">
+        <v>370</v>
+      </c>
+      <c r="E29" s="102" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="F29" s="102" t="n">
+        <v>64.09999999999999</v>
+      </c>
+      <c r="G29" s="73" t="n"/>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="B30" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C30" s="75" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D30" s="98" t="n">
+        <v>69</v>
+      </c>
+      <c r="E30" s="98" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="F30" s="98" t="n">
+        <v>12</v>
+      </c>
+      <c r="G30" s="77" t="n"/>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="B31" s="86" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="C31" s="86" t="inlineStr"/>
+      <c r="D31" s="86" t="n">
+        <v>577</v>
+      </c>
+      <c r="E31" s="86" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="F31" s="86" t="n">
+        <v>100</v>
+      </c>
+      <c r="G31" s="109" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B23:G23"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>